<commit_message>
Portada: velo blanco + marca de agua del logo, flechas naranja con hover blanco, hero +10px; inventario portada completado
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventario-fotos-web.xlsx
+++ b/inventario-fotos-web.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,8 +70,13 @@
       <color rgb="00C00000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -103,8 +108,13 @@
         <fgColor rgb="00F4F4F4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -126,11 +136,55 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -177,6 +231,23 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -543,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -568,7 +639,16 @@
           <t>Link carpeta central de fotos:</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1MgJ6f1yEm0SKYoHiM9TQy_7O3IbEHhax</t>
+        </is>
+      </c>
+      <c r="C2" s="18" t="n"/>
+      <c r="D2" s="18" t="n"/>
+      <c r="E2" s="18" t="n"/>
+      <c r="F2" s="18" t="n"/>
+      <c r="G2" s="19" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -652,22 +732,22 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>Inicio</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>Encabezado (hero)</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>Grupo formando la palabra "JUNTOS"</t>
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>Portada — carrusel (rotativa)</t>
+        </is>
+      </c>
+      <c r="D7" s="21" t="inlineStr">
+        <is>
+          <t>Grupo bajo arco "BIENVENIDOS" (panorámica)</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
@@ -675,26 +755,34 @@
           <t>Cargada</t>
         </is>
       </c>
-      <c r="F7" s="11" t="inlineStr"/>
-      <c r="G7" s="11" t="inlineStr"/>
+      <c r="F7" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G7" s="23" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1bpKGEEe5qZVCX2_WJ2bfcczSRdloF5gy/view</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="n">
+      <c r="A8" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>Inicio</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Servicios — card</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>Gymkanas productivas</t>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>Portada — carrusel (rotativa)</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>Campo con carpas de colores y actividades</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -702,26 +790,34 @@
           <t>Cargada</t>
         </is>
       </c>
-      <c r="F8" s="11" t="inlineStr"/>
-      <c r="G8" s="11" t="inlineStr"/>
+      <c r="F8" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/18gkDcpy2v4ajAHfLSjqStHPSv5znxVec/view</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="n">
+      <c r="A9" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>Inicio</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Servicios — card</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>Team building</t>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>Portada — carrusel (rotativa)</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>Bubble soccer en el campo</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
@@ -729,26 +825,34 @@
           <t>Cargada</t>
         </is>
       </c>
-      <c r="F9" s="11" t="inlineStr"/>
-      <c r="G9" s="11" t="inlineStr"/>
+      <c r="F9" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G9" s="23" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1IQIts1momeIJnvDenIN2V8zgI9Yuzu3I/view</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="n">
+      <c r="A10" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>Inicio</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>Servicios — card</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>Eventos privados</t>
+      <c r="C10" s="21" t="inlineStr">
+        <is>
+          <t>Portada — carrusel (rotativa)</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>Colaboradora campeona con trofeo</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
@@ -756,8 +860,16 @@
           <t>Cargada</t>
         </is>
       </c>
-      <c r="F10" s="11" t="inlineStr"/>
-      <c r="G10" s="11" t="inlineStr"/>
+      <c r="F10" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G10" s="23" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/11nmFeZH_GDXNDlBeqdOonSWJMttFoNm3/view</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n">
@@ -770,12 +882,12 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Un equipo unido — carrusel</t>
+          <t>Servicios — card</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Equipo de catering en evento corporativo</t>
+          <t>Gymkanas productivas</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -797,12 +909,12 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Un equipo unido — carrusel</t>
+          <t>Servicios — card</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Bingo corporativo con colaboradores</t>
+          <t>Team building</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
@@ -824,12 +936,12 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>Un equipo unido — carrusel</t>
+          <t>Servicios — card</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>Dinámica de disfraces gigantes en equipo</t>
+          <t>Eventos privados</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr">
@@ -856,7 +968,7 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>Colaboradora celebrando con trofeo</t>
+          <t>Equipo de catering en evento corporativo</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
@@ -883,7 +995,7 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Carpas de feria corporativa decoradas</t>
+          <t>Bingo corporativo con colaboradores</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr">
@@ -905,12 +1017,12 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Diferenciales</t>
+          <t>Un equipo unido — carrusel</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Actividad grupal al aire libre</t>
+          <t>Dinámica de disfraces gigantes en equipo</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
@@ -932,12 +1044,12 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Diferenciales</t>
+          <t>Un equipo unido — carrusel</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Colaboradores en dinámica de integración</t>
+          <t>Colaboradora celebrando con trofeo</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr">
@@ -959,12 +1071,12 @@
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Diferenciales</t>
+          <t>Un equipo unido — carrusel</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Colaboradores participando en actividad</t>
+          <t>Carpas de feria corporativa decoradas</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
@@ -991,7 +1103,7 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Dinámica lúdica en evento</t>
+          <t>Actividad grupal al aire libre</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
@@ -1018,7 +1130,7 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>Equipo celebrando en evento corporativo</t>
+          <t>Colaboradores en dinámica de integración</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
@@ -1045,7 +1157,7 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Equipo compartiendo en dinámica de integración</t>
+          <t>Colaboradores participando en actividad</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
@@ -1072,7 +1184,7 @@
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Equipo participando en gymkana</t>
+          <t>Dinámica lúdica en evento</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
@@ -1099,7 +1211,7 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Equipo trabajando junto en actividad</t>
+          <t>Equipo celebrando en evento corporativo</t>
         </is>
       </c>
       <c r="E23" s="10" t="inlineStr">
@@ -1111,25 +1223,25 @@
       <c r="G23" s="11" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="n">
+      <c r="A24" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="B24" s="13" t="inlineStr">
-        <is>
-          <t>Quiénes somos</t>
-        </is>
-      </c>
-      <c r="C24" s="13" t="inlineStr">
-        <is>
-          <t>Encabezado (carrusel)</t>
-        </is>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
-        <is>
-          <t>Fútbol burbuja corporativo</t>
-        </is>
-      </c>
-      <c r="E24" s="14" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Inicio</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Diferenciales</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Equipo compartiendo en dinámica de integración</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
         <is>
           <t>Cargada</t>
         </is>
@@ -1138,25 +1250,25 @@
       <c r="G24" s="11" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="n">
+      <c r="A25" s="8" t="n">
         <v>19</v>
       </c>
-      <c r="B25" s="13" t="inlineStr">
-        <is>
-          <t>Quiénes somos</t>
-        </is>
-      </c>
-      <c r="C25" s="13" t="inlineStr">
-        <is>
-          <t>Encabezado (carrusel)</t>
-        </is>
-      </c>
-      <c r="D25" s="13" t="inlineStr">
-        <is>
-          <t>Arco de bienvenida Gymkanas</t>
-        </is>
-      </c>
-      <c r="E25" s="14" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Inicio</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Diferenciales</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Equipo participando en gymkana</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
         <is>
           <t>Cargada</t>
         </is>
@@ -1165,25 +1277,25 @@
       <c r="G25" s="11" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="n">
+      <c r="A26" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="B26" s="13" t="inlineStr">
-        <is>
-          <t>Quiénes somos</t>
-        </is>
-      </c>
-      <c r="C26" s="13" t="inlineStr">
-        <is>
-          <t>Encabezado (carrusel)</t>
-        </is>
-      </c>
-      <c r="D26" s="13" t="inlineStr">
-        <is>
-          <t>Dinámica de disfraces corporativa</t>
-        </is>
-      </c>
-      <c r="E26" s="14" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Inicio</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Diferenciales</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>Equipo trabajando junto en actividad</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
         <is>
           <t>Cargada</t>
         </is>
@@ -1207,7 +1319,7 @@
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>Comparsa y batucada en evento</t>
+          <t>Fútbol burbuja corporativo</t>
         </is>
       </c>
       <c r="E27" s="14" t="inlineStr">
@@ -1229,12 +1341,12 @@
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Liderazgo</t>
+          <t>Encabezado (carrusel)</t>
         </is>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>Foto de la pestaña</t>
+          <t>Arco de bienvenida Gymkanas</t>
         </is>
       </c>
       <c r="E28" s="14" t="inlineStr">
@@ -1256,12 +1368,12 @@
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Productividad</t>
+          <t>Encabezado (carrusel)</t>
         </is>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>Foto de la pestaña</t>
+          <t>Dinámica de disfraces corporativa</t>
         </is>
       </c>
       <c r="E29" s="14" t="inlineStr">
@@ -1283,12 +1395,12 @@
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Engagement</t>
+          <t>Encabezado (carrusel)</t>
         </is>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Foto de la pestaña</t>
+          <t>Comparsa y batucada en evento</t>
         </is>
       </c>
       <c r="E30" s="14" t="inlineStr">
@@ -1310,7 +1422,7 @@
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Retención de talento</t>
+          <t>Superpoderes — Liderazgo</t>
         </is>
       </c>
       <c r="D31" s="13" t="inlineStr">
@@ -1337,12 +1449,12 @@
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Calidez humana</t>
+          <t>Superpoderes — Productividad</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>Equipo con cartel "Solo integrados..."</t>
+          <t>Foto de la pestaña</t>
         </is>
       </c>
       <c r="E32" s="14" t="inlineStr">
@@ -1354,25 +1466,25 @@
       <c r="G32" s="11" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="n">
+      <c r="A33" s="12" t="n">
         <v>27</v>
       </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>Servicios</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="inlineStr">
-        <is>
-          <t>Encabezado (carrusel)</t>
-        </is>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
-        <is>
-          <t>Fútbol burbuja corporativo</t>
-        </is>
-      </c>
-      <c r="E33" s="10" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>Quiénes somos</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>Superpoderes — Engagement</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>Foto de la pestaña</t>
+        </is>
+      </c>
+      <c r="E33" s="14" t="inlineStr">
         <is>
           <t>Cargada</t>
         </is>
@@ -1381,25 +1493,25 @@
       <c r="G33" s="11" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="n">
+      <c r="A34" s="12" t="n">
         <v>28</v>
       </c>
-      <c r="B34" s="9" t="inlineStr">
-        <is>
-          <t>Servicios</t>
-        </is>
-      </c>
-      <c r="C34" s="9" t="inlineStr">
-        <is>
-          <t>Encabezado (carrusel)</t>
-        </is>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
-        <is>
-          <t>Arco de bienvenida Gymkanas</t>
-        </is>
-      </c>
-      <c r="E34" s="10" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>Quiénes somos</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>Superpoderes — Retención de talento</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>Foto de la pestaña</t>
+        </is>
+      </c>
+      <c r="E34" s="14" t="inlineStr">
         <is>
           <t>Cargada</t>
         </is>
@@ -1408,25 +1520,25 @@
       <c r="G34" s="11" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="8" t="n">
+      <c r="A35" s="12" t="n">
         <v>29</v>
       </c>
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>Servicios</t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>Encabezado (carrusel)</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
-        <is>
-          <t>Dinámica de disfraces corporativa</t>
-        </is>
-      </c>
-      <c r="E35" s="10" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>Quiénes somos</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>Superpoderes — Calidez humana</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>Equipo con cartel "Solo integrados..."</t>
+        </is>
+      </c>
+      <c r="E35" s="14" t="inlineStr">
         <is>
           <t>Cargada</t>
         </is>
@@ -1450,7 +1562,7 @@
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Comparsa y batucada en evento</t>
+          <t>Fútbol burbuja corporativo</t>
         </is>
       </c>
       <c r="E36" s="10" t="inlineStr">
@@ -1472,12 +1584,12 @@
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Gymkanas productivas</t>
+          <t>Encabezado (carrusel)</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Foto de la experiencia</t>
+          <t>Arco de bienvenida Gymkanas</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
@@ -1499,12 +1611,12 @@
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Team building</t>
+          <t>Encabezado (carrusel)</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Foto de la experiencia</t>
+          <t>Dinámica de disfraces corporativa</t>
         </is>
       </c>
       <c r="E38" s="10" t="inlineStr">
@@ -1526,12 +1638,12 @@
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Bingo Show</t>
+          <t>Encabezado (carrusel)</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Foto de la experiencia</t>
+          <t>Comparsa y batucada en evento</t>
         </is>
       </c>
       <c r="E39" s="10" t="inlineStr">
@@ -1553,7 +1665,7 @@
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Juegos de feria</t>
+          <t>Pestaña — Gymkanas productivas</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
@@ -1580,7 +1692,7 @@
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Full Day</t>
+          <t>Pestaña — Team building</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
@@ -1607,7 +1719,7 @@
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Eventos privados</t>
+          <t>Pestaña — Bingo Show</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
@@ -1624,25 +1736,25 @@
       <c r="G42" s="11" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="12" t="n">
+      <c r="A43" s="8" t="n">
         <v>37</v>
       </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>Team building (subpágina)</t>
-        </is>
-      </c>
-      <c r="C43" s="13" t="inlineStr">
-        <is>
-          <t>Encabezado (carrusel horizontal)</t>
-        </is>
-      </c>
-      <c r="D43" s="13" t="inlineStr">
-        <is>
-          <t>Foto 1</t>
-        </is>
-      </c>
-      <c r="E43" s="14" t="inlineStr">
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>Pestaña — Juegos de feria</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>Foto de la experiencia</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="inlineStr">
         <is>
           <t>Cargada</t>
         </is>
@@ -1651,25 +1763,25 @@
       <c r="G43" s="11" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="12" t="n">
+      <c r="A44" s="8" t="n">
         <v>38</v>
       </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>Team building (subpágina)</t>
-        </is>
-      </c>
-      <c r="C44" s="13" t="inlineStr">
-        <is>
-          <t>Encabezado (carrusel horizontal)</t>
-        </is>
-      </c>
-      <c r="D44" s="13" t="inlineStr">
-        <is>
-          <t>Foto 2</t>
-        </is>
-      </c>
-      <c r="E44" s="14" t="inlineStr">
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>Pestaña — Full Day</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>Foto de la experiencia</t>
+        </is>
+      </c>
+      <c r="E44" s="10" t="inlineStr">
         <is>
           <t>Cargada</t>
         </is>
@@ -1678,25 +1790,25 @@
       <c r="G44" s="11" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="12" t="n">
+      <c r="A45" s="8" t="n">
         <v>39</v>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>Team building (subpágina)</t>
-        </is>
-      </c>
-      <c r="C45" s="13" t="inlineStr">
-        <is>
-          <t>Encabezado (carrusel horizontal)</t>
-        </is>
-      </c>
-      <c r="D45" s="13" t="inlineStr">
-        <is>
-          <t>Foto 3</t>
-        </is>
-      </c>
-      <c r="E45" s="14" t="inlineStr">
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Pestaña — Eventos privados</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>Foto de la experiencia</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="inlineStr">
         <is>
           <t>Cargada</t>
         </is>
@@ -1720,7 +1832,7 @@
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
-          <t>Foto 4</t>
+          <t>Foto 1</t>
         </is>
       </c>
       <c r="E46" s="14" t="inlineStr">
@@ -1747,7 +1859,7 @@
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>Foto 5</t>
+          <t>Foto 2</t>
         </is>
       </c>
       <c r="E47" s="14" t="inlineStr">
@@ -1769,12 +1881,12 @@
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>En qué consiste (card vertical)</t>
+          <t>Encabezado (carrusel horizontal)</t>
         </is>
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>Foto 1</t>
+          <t>Foto 3</t>
         </is>
       </c>
       <c r="E48" s="14" t="inlineStr">
@@ -1796,12 +1908,12 @@
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>En qué consiste (card vertical)</t>
+          <t>Encabezado (carrusel horizontal)</t>
         </is>
       </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
-          <t>Foto 2</t>
+          <t>Foto 4</t>
         </is>
       </c>
       <c r="E49" s="14" t="inlineStr">
@@ -1823,12 +1935,12 @@
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Galería "en acción" (carrusel)</t>
+          <t>Encabezado (carrusel horizontal)</t>
         </is>
       </c>
       <c r="D50" s="13" t="inlineStr">
         <is>
-          <t>Foto 1</t>
+          <t>Foto 5</t>
         </is>
       </c>
       <c r="E50" s="14" t="inlineStr">
@@ -1850,12 +1962,12 @@
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>Galería "en acción" (carrusel)</t>
+          <t>En qué consiste (card vertical)</t>
         </is>
       </c>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>Foto 2</t>
+          <t>Foto 1</t>
         </is>
       </c>
       <c r="E51" s="14" t="inlineStr">
@@ -1877,12 +1989,12 @@
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>Galería "en acción" (carrusel)</t>
+          <t>En qué consiste (card vertical)</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>Foto 3</t>
+          <t>Foto 2</t>
         </is>
       </c>
       <c r="E52" s="14" t="inlineStr">
@@ -1909,7 +2021,7 @@
       </c>
       <c r="D53" s="13" t="inlineStr">
         <is>
-          <t>Foto 4</t>
+          <t>Foto 1</t>
         </is>
       </c>
       <c r="E53" s="14" t="inlineStr">
@@ -1921,106 +2033,106 @@
       <c r="G53" s="11" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="8" t="n">
+      <c r="A54" s="12" t="n">
         <v>48</v>
       </c>
-      <c r="B54" s="9" t="inlineStr">
-        <is>
-          <t>Gymkanas productivas (subpágina)</t>
-        </is>
-      </c>
-      <c r="C54" s="9" t="inlineStr">
-        <is>
-          <t>Encabezado (hero)</t>
-        </is>
-      </c>
-      <c r="D54" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E54" s="15" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>Team building (subpágina)</t>
+        </is>
+      </c>
+      <c r="C54" s="13" t="inlineStr">
+        <is>
+          <t>Galería "en acción" (carrusel)</t>
+        </is>
+      </c>
+      <c r="D54" s="13" t="inlineStr">
+        <is>
+          <t>Foto 2</t>
+        </is>
+      </c>
+      <c r="E54" s="14" t="inlineStr">
+        <is>
+          <t>Cargada</t>
         </is>
       </c>
       <c r="F54" s="11" t="inlineStr"/>
       <c r="G54" s="11" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="8" t="n">
+      <c r="A55" s="12" t="n">
         <v>49</v>
       </c>
-      <c r="B55" s="9" t="inlineStr">
-        <is>
-          <t>Gymkanas productivas (subpágina)</t>
-        </is>
-      </c>
-      <c r="C55" s="9" t="inlineStr">
-        <is>
-          <t>En qué consiste (card)</t>
-        </is>
-      </c>
-      <c r="D55" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E55" s="15" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>Team building (subpágina)</t>
+        </is>
+      </c>
+      <c r="C55" s="13" t="inlineStr">
+        <is>
+          <t>Galería "en acción" (carrusel)</t>
+        </is>
+      </c>
+      <c r="D55" s="13" t="inlineStr">
+        <is>
+          <t>Foto 3</t>
+        </is>
+      </c>
+      <c r="E55" s="14" t="inlineStr">
+        <is>
+          <t>Cargada</t>
         </is>
       </c>
       <c r="F55" s="11" t="inlineStr"/>
       <c r="G55" s="11" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="8" t="n">
+      <c r="A56" s="12" t="n">
         <v>50</v>
       </c>
-      <c r="B56" s="9" t="inlineStr">
-        <is>
-          <t>Gymkanas productivas (subpágina)</t>
-        </is>
-      </c>
-      <c r="C56" s="9" t="inlineStr">
-        <is>
-          <t>Galería "en vivo"</t>
-        </is>
-      </c>
-      <c r="D56" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E56" s="15" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>Team building (subpágina)</t>
+        </is>
+      </c>
+      <c r="C56" s="13" t="inlineStr">
+        <is>
+          <t>Galería "en acción" (carrusel)</t>
+        </is>
+      </c>
+      <c r="D56" s="13" t="inlineStr">
+        <is>
+          <t>Foto 4</t>
+        </is>
+      </c>
+      <c r="E56" s="14" t="inlineStr">
+        <is>
+          <t>Cargada</t>
         </is>
       </c>
       <c r="F56" s="11" t="inlineStr"/>
       <c r="G56" s="11" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="12" t="n">
+      <c r="A57" s="8" t="n">
         <v>51</v>
       </c>
-      <c r="B57" s="13" t="inlineStr">
-        <is>
-          <t>Bingo Show (subpágina)</t>
-        </is>
-      </c>
-      <c r="C57" s="13" t="inlineStr">
+      <c r="B57" s="9" t="inlineStr">
+        <is>
+          <t>Gymkanas productivas (subpágina)</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
         <is>
           <t>Encabezado (hero)</t>
         </is>
       </c>
-      <c r="D57" s="13" t="inlineStr">
+      <c r="D57" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E57" s="16" t="inlineStr">
+      <c r="E57" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2029,25 +2141,25 @@
       <c r="G57" s="11" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="12" t="n">
+      <c r="A58" s="8" t="n">
         <v>52</v>
       </c>
-      <c r="B58" s="13" t="inlineStr">
-        <is>
-          <t>Bingo Show (subpágina)</t>
-        </is>
-      </c>
-      <c r="C58" s="13" t="inlineStr">
+      <c r="B58" s="9" t="inlineStr">
+        <is>
+          <t>Gymkanas productivas (subpágina)</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr">
         <is>
           <t>En qué consiste (card)</t>
         </is>
       </c>
-      <c r="D58" s="13" t="inlineStr">
+      <c r="D58" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E58" s="16" t="inlineStr">
+      <c r="E58" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2056,25 +2168,25 @@
       <c r="G58" s="11" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="12" t="n">
+      <c r="A59" s="8" t="n">
         <v>53</v>
       </c>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t>Bingo Show (subpágina)</t>
-        </is>
-      </c>
-      <c r="C59" s="13" t="inlineStr">
+      <c r="B59" s="9" t="inlineStr">
+        <is>
+          <t>Gymkanas productivas (subpágina)</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
         <is>
           <t>Galería "en vivo"</t>
         </is>
       </c>
-      <c r="D59" s="13" t="inlineStr">
+      <c r="D59" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E59" s="16" t="inlineStr">
+      <c r="E59" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2083,25 +2195,25 @@
       <c r="G59" s="11" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="8" t="n">
+      <c r="A60" s="12" t="n">
         <v>54</v>
       </c>
-      <c r="B60" s="9" t="inlineStr">
-        <is>
-          <t>Juegos de feria (subpágina)</t>
-        </is>
-      </c>
-      <c r="C60" s="9" t="inlineStr">
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>Bingo Show (subpágina)</t>
+        </is>
+      </c>
+      <c r="C60" s="13" t="inlineStr">
         <is>
           <t>Encabezado (hero)</t>
         </is>
       </c>
-      <c r="D60" s="9" t="inlineStr">
+      <c r="D60" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E60" s="15" t="inlineStr">
+      <c r="E60" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2110,25 +2222,25 @@
       <c r="G60" s="11" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="8" t="n">
+      <c r="A61" s="12" t="n">
         <v>55</v>
       </c>
-      <c r="B61" s="9" t="inlineStr">
-        <is>
-          <t>Juegos de feria (subpágina)</t>
-        </is>
-      </c>
-      <c r="C61" s="9" t="inlineStr">
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>Bingo Show (subpágina)</t>
+        </is>
+      </c>
+      <c r="C61" s="13" t="inlineStr">
         <is>
           <t>En qué consiste (card)</t>
         </is>
       </c>
-      <c r="D61" s="9" t="inlineStr">
+      <c r="D61" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E61" s="15" t="inlineStr">
+      <c r="E61" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2137,25 +2249,25 @@
       <c r="G61" s="11" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="8" t="n">
+      <c r="A62" s="12" t="n">
         <v>56</v>
       </c>
-      <c r="B62" s="9" t="inlineStr">
-        <is>
-          <t>Juegos de feria (subpágina)</t>
-        </is>
-      </c>
-      <c r="C62" s="9" t="inlineStr">
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>Bingo Show (subpágina)</t>
+        </is>
+      </c>
+      <c r="C62" s="13" t="inlineStr">
         <is>
           <t>Galería "en vivo"</t>
         </is>
       </c>
-      <c r="D62" s="9" t="inlineStr">
+      <c r="D62" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E62" s="15" t="inlineStr">
+      <c r="E62" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2164,25 +2276,25 @@
       <c r="G62" s="11" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="12" t="n">
+      <c r="A63" s="8" t="n">
         <v>57</v>
       </c>
-      <c r="B63" s="13" t="inlineStr">
-        <is>
-          <t>Full Day (subpágina)</t>
-        </is>
-      </c>
-      <c r="C63" s="13" t="inlineStr">
+      <c r="B63" s="9" t="inlineStr">
+        <is>
+          <t>Juegos de feria (subpágina)</t>
+        </is>
+      </c>
+      <c r="C63" s="9" t="inlineStr">
         <is>
           <t>Encabezado (hero)</t>
         </is>
       </c>
-      <c r="D63" s="13" t="inlineStr">
+      <c r="D63" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E63" s="16" t="inlineStr">
+      <c r="E63" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2191,25 +2303,25 @@
       <c r="G63" s="11" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="12" t="n">
+      <c r="A64" s="8" t="n">
         <v>58</v>
       </c>
-      <c r="B64" s="13" t="inlineStr">
-        <is>
-          <t>Full Day (subpágina)</t>
-        </is>
-      </c>
-      <c r="C64" s="13" t="inlineStr">
+      <c r="B64" s="9" t="inlineStr">
+        <is>
+          <t>Juegos de feria (subpágina)</t>
+        </is>
+      </c>
+      <c r="C64" s="9" t="inlineStr">
         <is>
           <t>En qué consiste (card)</t>
         </is>
       </c>
-      <c r="D64" s="13" t="inlineStr">
+      <c r="D64" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E64" s="16" t="inlineStr">
+      <c r="E64" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2218,25 +2330,25 @@
       <c r="G64" s="11" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="12" t="n">
+      <c r="A65" s="8" t="n">
         <v>59</v>
       </c>
-      <c r="B65" s="13" t="inlineStr">
-        <is>
-          <t>Full Day (subpágina)</t>
-        </is>
-      </c>
-      <c r="C65" s="13" t="inlineStr">
+      <c r="B65" s="9" t="inlineStr">
+        <is>
+          <t>Juegos de feria (subpágina)</t>
+        </is>
+      </c>
+      <c r="C65" s="9" t="inlineStr">
         <is>
           <t>Galería "en vivo"</t>
         </is>
       </c>
-      <c r="D65" s="13" t="inlineStr">
+      <c r="D65" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E65" s="16" t="inlineStr">
+      <c r="E65" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2245,25 +2357,25 @@
       <c r="G65" s="11" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="8" t="n">
+      <c r="A66" s="12" t="n">
         <v>60</v>
       </c>
-      <c r="B66" s="9" t="inlineStr">
-        <is>
-          <t>Eventos privados (subpágina)</t>
-        </is>
-      </c>
-      <c r="C66" s="9" t="inlineStr">
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>Full Day (subpágina)</t>
+        </is>
+      </c>
+      <c r="C66" s="13" t="inlineStr">
         <is>
           <t>Encabezado (hero)</t>
         </is>
       </c>
-      <c r="D66" s="9" t="inlineStr">
+      <c r="D66" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E66" s="15" t="inlineStr">
+      <c r="E66" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2272,25 +2384,25 @@
       <c r="G66" s="11" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="8" t="n">
+      <c r="A67" s="12" t="n">
         <v>61</v>
       </c>
-      <c r="B67" s="9" t="inlineStr">
-        <is>
-          <t>Eventos privados (subpágina)</t>
-        </is>
-      </c>
-      <c r="C67" s="9" t="inlineStr">
+      <c r="B67" s="13" t="inlineStr">
+        <is>
+          <t>Full Day (subpágina)</t>
+        </is>
+      </c>
+      <c r="C67" s="13" t="inlineStr">
         <is>
           <t>En qué consiste (card)</t>
         </is>
       </c>
-      <c r="D67" s="9" t="inlineStr">
+      <c r="D67" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E67" s="15" t="inlineStr">
+      <c r="E67" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2299,31 +2411,112 @@
       <c r="G67" s="11" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="8" t="n">
+      <c r="A68" s="12" t="n">
         <v>62</v>
       </c>
-      <c r="B68" s="9" t="inlineStr">
-        <is>
-          <t>Eventos privados (subpágina)</t>
-        </is>
-      </c>
-      <c r="C68" s="9" t="inlineStr">
+      <c r="B68" s="13" t="inlineStr">
+        <is>
+          <t>Full Day (subpágina)</t>
+        </is>
+      </c>
+      <c r="C68" s="13" t="inlineStr">
         <is>
           <t>Galería "en vivo"</t>
         </is>
       </c>
-      <c r="D68" s="9" t="inlineStr">
+      <c r="D68" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E68" s="15" t="inlineStr">
+      <c r="E68" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
       <c r="F68" s="11" t="inlineStr"/>
       <c r="G68" s="11" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="n">
+        <v>63</v>
+      </c>
+      <c r="B69" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C69" s="9" t="inlineStr">
+        <is>
+          <t>Encabezado (hero)</t>
+        </is>
+      </c>
+      <c r="D69" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E69" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F69" s="11" t="inlineStr"/>
+      <c r="G69" s="11" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="n">
+        <v>64</v>
+      </c>
+      <c r="B70" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C70" s="9" t="inlineStr">
+        <is>
+          <t>En qué consiste (card)</t>
+        </is>
+      </c>
+      <c r="D70" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E70" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F70" s="11" t="inlineStr"/>
+      <c r="G70" s="11" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="B71" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C71" s="9" t="inlineStr">
+        <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D71" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E71" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F71" s="11" t="inlineStr"/>
+      <c r="G71" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Home: seccion 'Un equipo unido' (filosofia) en naranja; quita foto del trofeo del carrusel; inventario seccion carrusel actualizado
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventario-fotos-web.xlsx
+++ b/inventario-fotos-web.xlsx
@@ -184,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -247,6 +247,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -614,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -963,12 +966,12 @@
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Un equipo unido — carrusel</t>
+          <t>¿Diseñamos juntos una experiencia extraordinaria?</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>Equipo de catering en evento corporativo</t>
+          <t>Equipo de catering (mozos y chef) junto a mesa de platos servidos</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
@@ -976,8 +979,16 @@
           <t>Cargada</t>
         </is>
       </c>
-      <c r="F14" s="11" t="inlineStr"/>
-      <c r="G14" s="11" t="inlineStr"/>
+      <c r="F14" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G14" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1CpiI8EKPfkVF_xjyozKN7ZMyFYGNK5xZ</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n">
@@ -990,7 +1001,7 @@
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Un equipo unido — carrusel</t>
+          <t>¿Diseñamos juntos una experiencia extraordinaria?</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
@@ -1003,8 +1014,16 @@
           <t>Cargada</t>
         </is>
       </c>
-      <c r="F15" s="11" t="inlineStr"/>
-      <c r="G15" s="11" t="inlineStr"/>
+      <c r="F15" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G15" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1CpiI8EKPfkVF_xjyozKN7ZMyFYGNK5xZ</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n">
@@ -1017,12 +1036,12 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Un equipo unido — carrusel</t>
+          <t>¿Diseñamos juntos una experiencia extraordinaria?</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Dinámica de disfraces gigantes en equipo</t>
+          <t>Dinámica de disfraces / pantalones gigantes en equipo</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
@@ -1030,8 +1049,16 @@
           <t>Cargada</t>
         </is>
       </c>
-      <c r="F16" s="11" t="inlineStr"/>
-      <c r="G16" s="11" t="inlineStr"/>
+      <c r="F16" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G16" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1CpiI8EKPfkVF_xjyozKN7ZMyFYGNK5xZ</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n">
@@ -1044,12 +1071,12 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Un equipo unido — carrusel</t>
+          <t>¿Diseñamos juntos una experiencia extraordinaria?</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Colaboradora celebrando con trofeo</t>
+          <t>Carpas de feria corporativa decoradas</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr">
@@ -1057,8 +1084,16 @@
           <t>Cargada</t>
         </is>
       </c>
-      <c r="F17" s="11" t="inlineStr"/>
-      <c r="G17" s="11" t="inlineStr"/>
+      <c r="F17" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G17" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1CpiI8EKPfkVF_xjyozKN7ZMyFYGNK5xZ</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
@@ -1071,12 +1106,12 @@
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Un equipo unido — carrusel</t>
+          <t>Diferenciales</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Carpas de feria corporativa decoradas</t>
+          <t>Actividad grupal al aire libre</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
@@ -1103,7 +1138,7 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Actividad grupal al aire libre</t>
+          <t>Colaboradores en dinámica de integración</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
@@ -1130,7 +1165,7 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>Colaboradores en dinámica de integración</t>
+          <t>Colaboradores participando en actividad</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
@@ -1157,7 +1192,7 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Colaboradores participando en actividad</t>
+          <t>Dinámica lúdica en evento</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
@@ -1184,7 +1219,7 @@
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Dinámica lúdica en evento</t>
+          <t>Equipo celebrando en evento corporativo</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
@@ -1211,7 +1246,7 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Equipo celebrando en evento corporativo</t>
+          <t>Equipo compartiendo en dinámica de integración</t>
         </is>
       </c>
       <c r="E23" s="10" t="inlineStr">
@@ -1238,7 +1273,7 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Equipo compartiendo en dinámica de integración</t>
+          <t>Equipo participando en gymkana</t>
         </is>
       </c>
       <c r="E24" s="10" t="inlineStr">
@@ -1265,7 +1300,7 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Equipo participando en gymkana</t>
+          <t>Equipo trabajando junto en actividad</t>
         </is>
       </c>
       <c r="E25" s="10" t="inlineStr">
@@ -1277,25 +1312,25 @@
       <c r="G25" s="11" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="n">
+      <c r="A26" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>Inicio</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>Diferenciales</t>
-        </is>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>Equipo trabajando junto en actividad</t>
-        </is>
-      </c>
-      <c r="E26" s="10" t="inlineStr">
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>Quiénes somos</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>Encabezado (carrusel)</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>Fútbol burbuja corporativo</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
         <is>
           <t>Cargada</t>
         </is>
@@ -1319,7 +1354,7 @@
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>Fútbol burbuja corporativo</t>
+          <t>Arco de bienvenida Gymkanas</t>
         </is>
       </c>
       <c r="E27" s="14" t="inlineStr">
@@ -1346,7 +1381,7 @@
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>Arco de bienvenida Gymkanas</t>
+          <t>Dinámica de disfraces corporativa</t>
         </is>
       </c>
       <c r="E28" s="14" t="inlineStr">
@@ -1373,7 +1408,7 @@
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>Dinámica de disfraces corporativa</t>
+          <t>Comparsa y batucada en evento</t>
         </is>
       </c>
       <c r="E29" s="14" t="inlineStr">
@@ -1395,12 +1430,12 @@
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Encabezado (carrusel)</t>
+          <t>Superpoderes — Liderazgo</t>
         </is>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Comparsa y batucada en evento</t>
+          <t>Foto de la pestaña</t>
         </is>
       </c>
       <c r="E30" s="14" t="inlineStr">
@@ -1422,7 +1457,7 @@
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Liderazgo</t>
+          <t>Superpoderes — Productividad</t>
         </is>
       </c>
       <c r="D31" s="13" t="inlineStr">
@@ -1449,7 +1484,7 @@
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Productividad</t>
+          <t>Superpoderes — Engagement</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
@@ -1476,7 +1511,7 @@
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Engagement</t>
+          <t>Superpoderes — Retención de talento</t>
         </is>
       </c>
       <c r="D33" s="13" t="inlineStr">
@@ -1503,12 +1538,12 @@
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Retención de talento</t>
+          <t>Superpoderes — Calidez humana</t>
         </is>
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>Foto de la pestaña</t>
+          <t>Equipo con cartel "Solo integrados..."</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
@@ -1520,25 +1555,25 @@
       <c r="G34" s="11" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="12" t="n">
+      <c r="A35" s="8" t="n">
         <v>29</v>
       </c>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>Quiénes somos</t>
-        </is>
-      </c>
-      <c r="C35" s="13" t="inlineStr">
-        <is>
-          <t>Superpoderes — Calidez humana</t>
-        </is>
-      </c>
-      <c r="D35" s="13" t="inlineStr">
-        <is>
-          <t>Equipo con cartel "Solo integrados..."</t>
-        </is>
-      </c>
-      <c r="E35" s="14" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Encabezado (carrusel)</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>Fútbol burbuja corporativo</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
         <is>
           <t>Cargada</t>
         </is>
@@ -1562,7 +1597,7 @@
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Fútbol burbuja corporativo</t>
+          <t>Arco de bienvenida Gymkanas</t>
         </is>
       </c>
       <c r="E36" s="10" t="inlineStr">
@@ -1589,7 +1624,7 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Arco de bienvenida Gymkanas</t>
+          <t>Dinámica de disfraces corporativa</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
@@ -1616,7 +1651,7 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Dinámica de disfraces corporativa</t>
+          <t>Comparsa y batucada en evento</t>
         </is>
       </c>
       <c r="E38" s="10" t="inlineStr">
@@ -1638,12 +1673,12 @@
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Encabezado (carrusel)</t>
+          <t>Pestaña — Gymkanas productivas</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Comparsa y batucada en evento</t>
+          <t>Foto de la experiencia</t>
         </is>
       </c>
       <c r="E39" s="10" t="inlineStr">
@@ -1665,7 +1700,7 @@
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Gymkanas productivas</t>
+          <t>Pestaña — Team building</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
@@ -1692,7 +1727,7 @@
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Team building</t>
+          <t>Pestaña — Bingo Show</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
@@ -1719,7 +1754,7 @@
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Bingo Show</t>
+          <t>Pestaña — Juegos de feria</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
@@ -1746,7 +1781,7 @@
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Juegos de feria</t>
+          <t>Pestaña — Full Day</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
@@ -1773,7 +1808,7 @@
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Full Day</t>
+          <t>Pestaña — Eventos privados</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
@@ -1790,25 +1825,25 @@
       <c r="G44" s="11" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="8" t="n">
+      <c r="A45" s="12" t="n">
         <v>39</v>
       </c>
-      <c r="B45" s="9" t="inlineStr">
-        <is>
-          <t>Servicios</t>
-        </is>
-      </c>
-      <c r="C45" s="9" t="inlineStr">
-        <is>
-          <t>Pestaña — Eventos privados</t>
-        </is>
-      </c>
-      <c r="D45" s="9" t="inlineStr">
-        <is>
-          <t>Foto de la experiencia</t>
-        </is>
-      </c>
-      <c r="E45" s="10" t="inlineStr">
+      <c r="B45" s="13" t="inlineStr">
+        <is>
+          <t>Team building (subpágina)</t>
+        </is>
+      </c>
+      <c r="C45" s="13" t="inlineStr">
+        <is>
+          <t>Encabezado (carrusel horizontal)</t>
+        </is>
+      </c>
+      <c r="D45" s="13" t="inlineStr">
+        <is>
+          <t>Foto 1</t>
+        </is>
+      </c>
+      <c r="E45" s="14" t="inlineStr">
         <is>
           <t>Cargada</t>
         </is>
@@ -1832,7 +1867,7 @@
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
-          <t>Foto 1</t>
+          <t>Foto 2</t>
         </is>
       </c>
       <c r="E46" s="14" t="inlineStr">
@@ -1859,7 +1894,7 @@
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>Foto 2</t>
+          <t>Foto 3</t>
         </is>
       </c>
       <c r="E47" s="14" t="inlineStr">
@@ -1886,7 +1921,7 @@
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>Foto 3</t>
+          <t>Foto 4</t>
         </is>
       </c>
       <c r="E48" s="14" t="inlineStr">
@@ -1913,7 +1948,7 @@
       </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
-          <t>Foto 4</t>
+          <t>Foto 5</t>
         </is>
       </c>
       <c r="E49" s="14" t="inlineStr">
@@ -1935,12 +1970,12 @@
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Encabezado (carrusel horizontal)</t>
+          <t>En qué consiste (card vertical)</t>
         </is>
       </c>
       <c r="D50" s="13" t="inlineStr">
         <is>
-          <t>Foto 5</t>
+          <t>Foto 1</t>
         </is>
       </c>
       <c r="E50" s="14" t="inlineStr">
@@ -1967,7 +2002,7 @@
       </c>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>Foto 1</t>
+          <t>Foto 2</t>
         </is>
       </c>
       <c r="E51" s="14" t="inlineStr">
@@ -1989,12 +2024,12 @@
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>En qué consiste (card vertical)</t>
+          <t>Galería "en acción" (carrusel)</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>Foto 2</t>
+          <t>Foto 1</t>
         </is>
       </c>
       <c r="E52" s="14" t="inlineStr">
@@ -2021,7 +2056,7 @@
       </c>
       <c r="D53" s="13" t="inlineStr">
         <is>
-          <t>Foto 1</t>
+          <t>Foto 2</t>
         </is>
       </c>
       <c r="E53" s="14" t="inlineStr">
@@ -2048,7 +2083,7 @@
       </c>
       <c r="D54" s="13" t="inlineStr">
         <is>
-          <t>Foto 2</t>
+          <t>Foto 3</t>
         </is>
       </c>
       <c r="E54" s="14" t="inlineStr">
@@ -2075,7 +2110,7 @@
       </c>
       <c r="D55" s="13" t="inlineStr">
         <is>
-          <t>Foto 3</t>
+          <t>Foto 4</t>
         </is>
       </c>
       <c r="E55" s="14" t="inlineStr">
@@ -2087,27 +2122,27 @@
       <c r="G55" s="11" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="12" t="n">
+      <c r="A56" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="B56" s="13" t="inlineStr">
-        <is>
-          <t>Team building (subpágina)</t>
-        </is>
-      </c>
-      <c r="C56" s="13" t="inlineStr">
-        <is>
-          <t>Galería "en acción" (carrusel)</t>
-        </is>
-      </c>
-      <c r="D56" s="13" t="inlineStr">
-        <is>
-          <t>Foto 4</t>
-        </is>
-      </c>
-      <c r="E56" s="14" t="inlineStr">
-        <is>
-          <t>Cargada</t>
+      <c r="B56" s="9" t="inlineStr">
+        <is>
+          <t>Gymkanas productivas (subpágina)</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>Encabezado (hero)</t>
+        </is>
+      </c>
+      <c r="D56" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E56" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F56" s="11" t="inlineStr"/>
@@ -2124,7 +2159,7 @@
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>Encabezado (hero)</t>
+          <t>En qué consiste (card)</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
@@ -2151,7 +2186,7 @@
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>En qué consiste (card)</t>
+          <t>Galería "en vivo"</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
@@ -2168,25 +2203,25 @@
       <c r="G58" s="11" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="8" t="n">
+      <c r="A59" s="12" t="n">
         <v>53</v>
       </c>
-      <c r="B59" s="9" t="inlineStr">
-        <is>
-          <t>Gymkanas productivas (subpágina)</t>
-        </is>
-      </c>
-      <c r="C59" s="9" t="inlineStr">
-        <is>
-          <t>Galería "en vivo"</t>
-        </is>
-      </c>
-      <c r="D59" s="9" t="inlineStr">
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>Bingo Show (subpágina)</t>
+        </is>
+      </c>
+      <c r="C59" s="13" t="inlineStr">
+        <is>
+          <t>Encabezado (hero)</t>
+        </is>
+      </c>
+      <c r="D59" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E59" s="15" t="inlineStr">
+      <c r="E59" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2205,7 +2240,7 @@
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>Encabezado (hero)</t>
+          <t>En qué consiste (card)</t>
         </is>
       </c>
       <c r="D60" s="13" t="inlineStr">
@@ -2232,7 +2267,7 @@
       </c>
       <c r="C61" s="13" t="inlineStr">
         <is>
-          <t>En qué consiste (card)</t>
+          <t>Galería "en vivo"</t>
         </is>
       </c>
       <c r="D61" s="13" t="inlineStr">
@@ -2249,25 +2284,25 @@
       <c r="G61" s="11" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="12" t="n">
+      <c r="A62" s="8" t="n">
         <v>56</v>
       </c>
-      <c r="B62" s="13" t="inlineStr">
-        <is>
-          <t>Bingo Show (subpágina)</t>
-        </is>
-      </c>
-      <c r="C62" s="13" t="inlineStr">
-        <is>
-          <t>Galería "en vivo"</t>
-        </is>
-      </c>
-      <c r="D62" s="13" t="inlineStr">
+      <c r="B62" s="9" t="inlineStr">
+        <is>
+          <t>Juegos de feria (subpágina)</t>
+        </is>
+      </c>
+      <c r="C62" s="9" t="inlineStr">
+        <is>
+          <t>Encabezado (hero)</t>
+        </is>
+      </c>
+      <c r="D62" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E62" s="16" t="inlineStr">
+      <c r="E62" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2286,7 +2321,7 @@
       </c>
       <c r="C63" s="9" t="inlineStr">
         <is>
-          <t>Encabezado (hero)</t>
+          <t>En qué consiste (card)</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
@@ -2313,7 +2348,7 @@
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>En qué consiste (card)</t>
+          <t>Galería "en vivo"</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
@@ -2330,25 +2365,25 @@
       <c r="G64" s="11" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="8" t="n">
+      <c r="A65" s="12" t="n">
         <v>59</v>
       </c>
-      <c r="B65" s="9" t="inlineStr">
-        <is>
-          <t>Juegos de feria (subpágina)</t>
-        </is>
-      </c>
-      <c r="C65" s="9" t="inlineStr">
-        <is>
-          <t>Galería "en vivo"</t>
-        </is>
-      </c>
-      <c r="D65" s="9" t="inlineStr">
+      <c r="B65" s="13" t="inlineStr">
+        <is>
+          <t>Full Day (subpágina)</t>
+        </is>
+      </c>
+      <c r="C65" s="13" t="inlineStr">
+        <is>
+          <t>Encabezado (hero)</t>
+        </is>
+      </c>
+      <c r="D65" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E65" s="15" t="inlineStr">
+      <c r="E65" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2367,7 +2402,7 @@
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>Encabezado (hero)</t>
+          <t>En qué consiste (card)</t>
         </is>
       </c>
       <c r="D66" s="13" t="inlineStr">
@@ -2394,7 +2429,7 @@
       </c>
       <c r="C67" s="13" t="inlineStr">
         <is>
-          <t>En qué consiste (card)</t>
+          <t>Galería "en vivo"</t>
         </is>
       </c>
       <c r="D67" s="13" t="inlineStr">
@@ -2411,25 +2446,25 @@
       <c r="G67" s="11" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="12" t="n">
+      <c r="A68" s="8" t="n">
         <v>62</v>
       </c>
-      <c r="B68" s="13" t="inlineStr">
-        <is>
-          <t>Full Day (subpágina)</t>
-        </is>
-      </c>
-      <c r="C68" s="13" t="inlineStr">
-        <is>
-          <t>Galería "en vivo"</t>
-        </is>
-      </c>
-      <c r="D68" s="13" t="inlineStr">
+      <c r="B68" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C68" s="9" t="inlineStr">
+        <is>
+          <t>Encabezado (hero)</t>
+        </is>
+      </c>
+      <c r="D68" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E68" s="16" t="inlineStr">
+      <c r="E68" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2448,7 +2483,7 @@
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>Encabezado (hero)</t>
+          <t>En qué consiste (card)</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
@@ -2475,7 +2510,7 @@
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>En qué consiste (card)</t>
+          <t>Galería "en vivo"</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
@@ -2490,33 +2525,6 @@
       </c>
       <c r="F70" s="11" t="inlineStr"/>
       <c r="G70" s="11" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="8" t="n">
-        <v>65</v>
-      </c>
-      <c r="B71" s="9" t="inlineStr">
-        <is>
-          <t>Eventos privados (subpágina)</t>
-        </is>
-      </c>
-      <c r="C71" s="9" t="inlineStr">
-        <is>
-          <t>Galería "en vivo"</t>
-        </is>
-      </c>
-      <c r="D71" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E71" s="15" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F71" s="11" t="inlineStr"/>
-      <c r="G71" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Portada quienes-somos: 6 fotos nuevas con flechas + tira de logos (como home); footer Bingo transparente en todas las paginas; inventario QS + columna Observacion (marca imagenes IA)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventario-fotos-web.xlsx
+++ b/inventario-fotos-web.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,6 +74,14 @@
       <name val="Arial"/>
       <color rgb="00000000"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -184,7 +192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -252,6 +260,7 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -617,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -627,6 +636,7 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -696,6 +706,11 @@
           <t>Link de la foto</t>
         </is>
       </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Observación</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1327,7 +1342,7 @@
       </c>
       <c r="D26" s="13" t="inlineStr">
         <is>
-          <t>Fútbol burbuja corporativo</t>
+          <t>Colaboradores compartiendo en evento corporativo</t>
         </is>
       </c>
       <c r="E26" s="14" t="inlineStr">
@@ -1335,8 +1350,17 @@
           <t>Cargada</t>
         </is>
       </c>
-      <c r="F26" s="11" t="inlineStr"/>
-      <c r="G26" s="11" t="inlineStr"/>
+      <c r="F26" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G26" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1YutPNgTVrT9IIkybRK9farlrShKlAHCo</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="12" t="n">
@@ -1354,7 +1378,7 @@
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>Arco de bienvenida Gymkanas</t>
+          <t>Fútbol burbuja en el campo</t>
         </is>
       </c>
       <c r="E27" s="14" t="inlineStr">
@@ -1362,8 +1386,17 @@
           <t>Cargada</t>
         </is>
       </c>
-      <c r="F27" s="11" t="inlineStr"/>
-      <c r="G27" s="11" t="inlineStr"/>
+      <c r="F27" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G27" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1YutPNgTVrT9IIkybRK9farlrShKlAHCo</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="12" t="n">
@@ -1381,7 +1414,7 @@
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>Dinámica de disfraces corporativa</t>
+          <t>Batucada y comparsa corporativa</t>
         </is>
       </c>
       <c r="E28" s="14" t="inlineStr">
@@ -1389,8 +1422,21 @@
           <t>Cargada</t>
         </is>
       </c>
-      <c r="F28" s="11" t="inlineStr"/>
-      <c r="G28" s="11" t="inlineStr"/>
+      <c r="F28" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G28" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1YutPNgTVrT9IIkybRK9farlrShKlAHCo</t>
+        </is>
+      </c>
+      <c r="H28" s="25" t="inlineStr">
+        <is>
+          <t>Se ve irreal (imagen IA)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="12" t="n">
@@ -1408,7 +1454,7 @@
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>Comparsa y batucada en evento</t>
+          <t>Dinámica de disfraces en equipo</t>
         </is>
       </c>
       <c r="E29" s="14" t="inlineStr">
@@ -1416,8 +1462,21 @@
           <t>Cargada</t>
         </is>
       </c>
-      <c r="F29" s="11" t="inlineStr"/>
-      <c r="G29" s="11" t="inlineStr"/>
+      <c r="F29" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G29" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1YutPNgTVrT9IIkybRK9farlrShKlAHCo</t>
+        </is>
+      </c>
+      <c r="H29" s="25" t="inlineStr">
+        <is>
+          <t>Se ve irreal (imagen IA)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="12" t="n">
@@ -1430,12 +1489,12 @@
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Liderazgo</t>
+          <t>Encabezado (carrusel)</t>
         </is>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Foto de la pestaña</t>
+          <t>Comedor del evento — mesas tipo picnic</t>
         </is>
       </c>
       <c r="E30" s="14" t="inlineStr">
@@ -1443,8 +1502,17 @@
           <t>Cargada</t>
         </is>
       </c>
-      <c r="F30" s="11" t="inlineStr"/>
-      <c r="G30" s="11" t="inlineStr"/>
+      <c r="F30" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G30" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1YutPNgTVrT9IIkybRK9farlrShKlAHCo</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="12" t="n">
@@ -1457,12 +1525,12 @@
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Productividad</t>
+          <t>Encabezado (carrusel)</t>
         </is>
       </c>
       <c r="D31" s="13" t="inlineStr">
         <is>
-          <t>Foto de la pestaña</t>
+          <t>Estación de jugos y desayuno de feria</t>
         </is>
       </c>
       <c r="E31" s="14" t="inlineStr">
@@ -1470,8 +1538,17 @@
           <t>Cargada</t>
         </is>
       </c>
-      <c r="F31" s="11" t="inlineStr"/>
-      <c r="G31" s="11" t="inlineStr"/>
+      <c r="F31" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G31" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1YutPNgTVrT9IIkybRK9farlrShKlAHCo</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="12" t="n">
@@ -1484,7 +1561,7 @@
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Engagement</t>
+          <t>Superpoderes — Liderazgo</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
@@ -1511,7 +1588,7 @@
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Retención de talento</t>
+          <t>Superpoderes — Productividad</t>
         </is>
       </c>
       <c r="D33" s="13" t="inlineStr">
@@ -1538,12 +1615,12 @@
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Calidez humana</t>
+          <t>Superpoderes — Engagement</t>
         </is>
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>Equipo con cartel "Solo integrados..."</t>
+          <t>Foto de la pestaña</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
@@ -1555,25 +1632,25 @@
       <c r="G34" s="11" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="8" t="n">
+      <c r="A35" s="12" t="n">
         <v>29</v>
       </c>
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>Servicios</t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>Encabezado (carrusel)</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
-        <is>
-          <t>Fútbol burbuja corporativo</t>
-        </is>
-      </c>
-      <c r="E35" s="10" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>Quiénes somos</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>Superpoderes — Retención de talento</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>Foto de la pestaña</t>
+        </is>
+      </c>
+      <c r="E35" s="14" t="inlineStr">
         <is>
           <t>Cargada</t>
         </is>
@@ -1582,25 +1659,25 @@
       <c r="G35" s="11" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="n">
+      <c r="A36" s="12" t="n">
         <v>30</v>
       </c>
-      <c r="B36" s="9" t="inlineStr">
-        <is>
-          <t>Servicios</t>
-        </is>
-      </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>Encabezado (carrusel)</t>
-        </is>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>Arco de bienvenida Gymkanas</t>
-        </is>
-      </c>
-      <c r="E36" s="10" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Quiénes somos</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>Superpoderes — Calidez humana</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>Equipo con cartel "Solo integrados..."</t>
+        </is>
+      </c>
+      <c r="E36" s="14" t="inlineStr">
         <is>
           <t>Cargada</t>
         </is>
@@ -1624,7 +1701,7 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Dinámica de disfraces corporativa</t>
+          <t>Fútbol burbuja corporativo</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
@@ -1651,7 +1728,7 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Comparsa y batucada en evento</t>
+          <t>Arco de bienvenida Gymkanas</t>
         </is>
       </c>
       <c r="E38" s="10" t="inlineStr">
@@ -1673,12 +1750,12 @@
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Gymkanas productivas</t>
+          <t>Encabezado (carrusel)</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Foto de la experiencia</t>
+          <t>Dinámica de disfraces corporativa</t>
         </is>
       </c>
       <c r="E39" s="10" t="inlineStr">
@@ -1700,12 +1777,12 @@
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Team building</t>
+          <t>Encabezado (carrusel)</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Foto de la experiencia</t>
+          <t>Comparsa y batucada en evento</t>
         </is>
       </c>
       <c r="E40" s="10" t="inlineStr">
@@ -1727,7 +1804,7 @@
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Bingo Show</t>
+          <t>Pestaña — Gymkanas productivas</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
@@ -1754,7 +1831,7 @@
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Juegos de feria</t>
+          <t>Pestaña — Team building</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
@@ -1781,7 +1858,7 @@
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Full Day</t>
+          <t>Pestaña — Bingo Show</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
@@ -1808,7 +1885,7 @@
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Eventos privados</t>
+          <t>Pestaña — Juegos de feria</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
@@ -1825,25 +1902,25 @@
       <c r="G44" s="11" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="12" t="n">
+      <c r="A45" s="8" t="n">
         <v>39</v>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>Team building (subpágina)</t>
-        </is>
-      </c>
-      <c r="C45" s="13" t="inlineStr">
-        <is>
-          <t>Encabezado (carrusel horizontal)</t>
-        </is>
-      </c>
-      <c r="D45" s="13" t="inlineStr">
-        <is>
-          <t>Foto 1</t>
-        </is>
-      </c>
-      <c r="E45" s="14" t="inlineStr">
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Pestaña — Full Day</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>Foto de la experiencia</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="inlineStr">
         <is>
           <t>Cargada</t>
         </is>
@@ -1852,25 +1929,25 @@
       <c r="G45" s="11" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="12" t="n">
+      <c r="A46" s="8" t="n">
         <v>40</v>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>Team building (subpágina)</t>
-        </is>
-      </c>
-      <c r="C46" s="13" t="inlineStr">
-        <is>
-          <t>Encabezado (carrusel horizontal)</t>
-        </is>
-      </c>
-      <c r="D46" s="13" t="inlineStr">
-        <is>
-          <t>Foto 2</t>
-        </is>
-      </c>
-      <c r="E46" s="14" t="inlineStr">
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>Pestaña — Eventos privados</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>Foto de la experiencia</t>
+        </is>
+      </c>
+      <c r="E46" s="10" t="inlineStr">
         <is>
           <t>Cargada</t>
         </is>
@@ -1894,7 +1971,7 @@
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>Foto 3</t>
+          <t>Foto 1</t>
         </is>
       </c>
       <c r="E47" s="14" t="inlineStr">
@@ -1921,7 +1998,7 @@
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>Foto 4</t>
+          <t>Foto 2</t>
         </is>
       </c>
       <c r="E48" s="14" t="inlineStr">
@@ -1948,7 +2025,7 @@
       </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
-          <t>Foto 5</t>
+          <t>Foto 3</t>
         </is>
       </c>
       <c r="E49" s="14" t="inlineStr">
@@ -1970,12 +2047,12 @@
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>En qué consiste (card vertical)</t>
+          <t>Encabezado (carrusel horizontal)</t>
         </is>
       </c>
       <c r="D50" s="13" t="inlineStr">
         <is>
-          <t>Foto 1</t>
+          <t>Foto 4</t>
         </is>
       </c>
       <c r="E50" s="14" t="inlineStr">
@@ -1997,12 +2074,12 @@
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>En qué consiste (card vertical)</t>
+          <t>Encabezado (carrusel horizontal)</t>
         </is>
       </c>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>Foto 2</t>
+          <t>Foto 5</t>
         </is>
       </c>
       <c r="E51" s="14" t="inlineStr">
@@ -2024,7 +2101,7 @@
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>Galería "en acción" (carrusel)</t>
+          <t>En qué consiste (card vertical)</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
@@ -2051,7 +2128,7 @@
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>Galería "en acción" (carrusel)</t>
+          <t>En qué consiste (card vertical)</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
@@ -2083,7 +2160,7 @@
       </c>
       <c r="D54" s="13" t="inlineStr">
         <is>
-          <t>Foto 3</t>
+          <t>Foto 1</t>
         </is>
       </c>
       <c r="E54" s="14" t="inlineStr">
@@ -2110,7 +2187,7 @@
       </c>
       <c r="D55" s="13" t="inlineStr">
         <is>
-          <t>Foto 4</t>
+          <t>Foto 2</t>
         </is>
       </c>
       <c r="E55" s="14" t="inlineStr">
@@ -2122,54 +2199,54 @@
       <c r="G55" s="11" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="8" t="n">
+      <c r="A56" s="12" t="n">
         <v>50</v>
       </c>
-      <c r="B56" s="9" t="inlineStr">
-        <is>
-          <t>Gymkanas productivas (subpágina)</t>
-        </is>
-      </c>
-      <c r="C56" s="9" t="inlineStr">
-        <is>
-          <t>Encabezado (hero)</t>
-        </is>
-      </c>
-      <c r="D56" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E56" s="15" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>Team building (subpágina)</t>
+        </is>
+      </c>
+      <c r="C56" s="13" t="inlineStr">
+        <is>
+          <t>Galería "en acción" (carrusel)</t>
+        </is>
+      </c>
+      <c r="D56" s="13" t="inlineStr">
+        <is>
+          <t>Foto 3</t>
+        </is>
+      </c>
+      <c r="E56" s="14" t="inlineStr">
+        <is>
+          <t>Cargada</t>
         </is>
       </c>
       <c r="F56" s="11" t="inlineStr"/>
       <c r="G56" s="11" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="8" t="n">
+      <c r="A57" s="12" t="n">
         <v>51</v>
       </c>
-      <c r="B57" s="9" t="inlineStr">
-        <is>
-          <t>Gymkanas productivas (subpágina)</t>
-        </is>
-      </c>
-      <c r="C57" s="9" t="inlineStr">
-        <is>
-          <t>En qué consiste (card)</t>
-        </is>
-      </c>
-      <c r="D57" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E57" s="15" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>Team building (subpágina)</t>
+        </is>
+      </c>
+      <c r="C57" s="13" t="inlineStr">
+        <is>
+          <t>Galería "en acción" (carrusel)</t>
+        </is>
+      </c>
+      <c r="D57" s="13" t="inlineStr">
+        <is>
+          <t>Foto 4</t>
+        </is>
+      </c>
+      <c r="E57" s="14" t="inlineStr">
+        <is>
+          <t>Cargada</t>
         </is>
       </c>
       <c r="F57" s="11" t="inlineStr"/>
@@ -2186,7 +2263,7 @@
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>Galería "en vivo"</t>
+          <t>Encabezado (hero)</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
@@ -2203,25 +2280,25 @@
       <c r="G58" s="11" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="12" t="n">
+      <c r="A59" s="8" t="n">
         <v>53</v>
       </c>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t>Bingo Show (subpágina)</t>
-        </is>
-      </c>
-      <c r="C59" s="13" t="inlineStr">
-        <is>
-          <t>Encabezado (hero)</t>
-        </is>
-      </c>
-      <c r="D59" s="13" t="inlineStr">
+      <c r="B59" s="9" t="inlineStr">
+        <is>
+          <t>Gymkanas productivas (subpágina)</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>En qué consiste (card)</t>
+        </is>
+      </c>
+      <c r="D59" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E59" s="16" t="inlineStr">
+      <c r="E59" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2230,25 +2307,25 @@
       <c r="G59" s="11" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="12" t="n">
+      <c r="A60" s="8" t="n">
         <v>54</v>
       </c>
-      <c r="B60" s="13" t="inlineStr">
-        <is>
-          <t>Bingo Show (subpágina)</t>
-        </is>
-      </c>
-      <c r="C60" s="13" t="inlineStr">
-        <is>
-          <t>En qué consiste (card)</t>
-        </is>
-      </c>
-      <c r="D60" s="13" t="inlineStr">
+      <c r="B60" s="9" t="inlineStr">
+        <is>
+          <t>Gymkanas productivas (subpágina)</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D60" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E60" s="16" t="inlineStr">
+      <c r="E60" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2267,7 +2344,7 @@
       </c>
       <c r="C61" s="13" t="inlineStr">
         <is>
-          <t>Galería "en vivo"</t>
+          <t>Encabezado (hero)</t>
         </is>
       </c>
       <c r="D61" s="13" t="inlineStr">
@@ -2284,25 +2361,25 @@
       <c r="G61" s="11" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="8" t="n">
+      <c r="A62" s="12" t="n">
         <v>56</v>
       </c>
-      <c r="B62" s="9" t="inlineStr">
-        <is>
-          <t>Juegos de feria (subpágina)</t>
-        </is>
-      </c>
-      <c r="C62" s="9" t="inlineStr">
-        <is>
-          <t>Encabezado (hero)</t>
-        </is>
-      </c>
-      <c r="D62" s="9" t="inlineStr">
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>Bingo Show (subpágina)</t>
+        </is>
+      </c>
+      <c r="C62" s="13" t="inlineStr">
+        <is>
+          <t>En qué consiste (card)</t>
+        </is>
+      </c>
+      <c r="D62" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E62" s="15" t="inlineStr">
+      <c r="E62" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2311,25 +2388,25 @@
       <c r="G62" s="11" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="8" t="n">
+      <c r="A63" s="12" t="n">
         <v>57</v>
       </c>
-      <c r="B63" s="9" t="inlineStr">
-        <is>
-          <t>Juegos de feria (subpágina)</t>
-        </is>
-      </c>
-      <c r="C63" s="9" t="inlineStr">
-        <is>
-          <t>En qué consiste (card)</t>
-        </is>
-      </c>
-      <c r="D63" s="9" t="inlineStr">
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>Bingo Show (subpágina)</t>
+        </is>
+      </c>
+      <c r="C63" s="13" t="inlineStr">
+        <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D63" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E63" s="15" t="inlineStr">
+      <c r="E63" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2348,7 +2425,7 @@
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>Galería "en vivo"</t>
+          <t>Encabezado (hero)</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
@@ -2365,25 +2442,25 @@
       <c r="G64" s="11" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="12" t="n">
+      <c r="A65" s="8" t="n">
         <v>59</v>
       </c>
-      <c r="B65" s="13" t="inlineStr">
-        <is>
-          <t>Full Day (subpágina)</t>
-        </is>
-      </c>
-      <c r="C65" s="13" t="inlineStr">
-        <is>
-          <t>Encabezado (hero)</t>
-        </is>
-      </c>
-      <c r="D65" s="13" t="inlineStr">
+      <c r="B65" s="9" t="inlineStr">
+        <is>
+          <t>Juegos de feria (subpágina)</t>
+        </is>
+      </c>
+      <c r="C65" s="9" t="inlineStr">
+        <is>
+          <t>En qué consiste (card)</t>
+        </is>
+      </c>
+      <c r="D65" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E65" s="16" t="inlineStr">
+      <c r="E65" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2392,25 +2469,25 @@
       <c r="G65" s="11" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="12" t="n">
+      <c r="A66" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="B66" s="13" t="inlineStr">
-        <is>
-          <t>Full Day (subpágina)</t>
-        </is>
-      </c>
-      <c r="C66" s="13" t="inlineStr">
-        <is>
-          <t>En qué consiste (card)</t>
-        </is>
-      </c>
-      <c r="D66" s="13" t="inlineStr">
+      <c r="B66" s="9" t="inlineStr">
+        <is>
+          <t>Juegos de feria (subpágina)</t>
+        </is>
+      </c>
+      <c r="C66" s="9" t="inlineStr">
+        <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D66" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E66" s="16" t="inlineStr">
+      <c r="E66" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2429,7 +2506,7 @@
       </c>
       <c r="C67" s="13" t="inlineStr">
         <is>
-          <t>Galería "en vivo"</t>
+          <t>Encabezado (hero)</t>
         </is>
       </c>
       <c r="D67" s="13" t="inlineStr">
@@ -2446,25 +2523,25 @@
       <c r="G67" s="11" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="8" t="n">
+      <c r="A68" s="12" t="n">
         <v>62</v>
       </c>
-      <c r="B68" s="9" t="inlineStr">
-        <is>
-          <t>Eventos privados (subpágina)</t>
-        </is>
-      </c>
-      <c r="C68" s="9" t="inlineStr">
-        <is>
-          <t>Encabezado (hero)</t>
-        </is>
-      </c>
-      <c r="D68" s="9" t="inlineStr">
+      <c r="B68" s="13" t="inlineStr">
+        <is>
+          <t>Full Day (subpágina)</t>
+        </is>
+      </c>
+      <c r="C68" s="13" t="inlineStr">
+        <is>
+          <t>En qué consiste (card)</t>
+        </is>
+      </c>
+      <c r="D68" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E68" s="15" t="inlineStr">
+      <c r="E68" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2473,25 +2550,25 @@
       <c r="G68" s="11" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="8" t="n">
+      <c r="A69" s="12" t="n">
         <v>63</v>
       </c>
-      <c r="B69" s="9" t="inlineStr">
-        <is>
-          <t>Eventos privados (subpágina)</t>
-        </is>
-      </c>
-      <c r="C69" s="9" t="inlineStr">
-        <is>
-          <t>En qué consiste (card)</t>
-        </is>
-      </c>
-      <c r="D69" s="9" t="inlineStr">
+      <c r="B69" s="13" t="inlineStr">
+        <is>
+          <t>Full Day (subpágina)</t>
+        </is>
+      </c>
+      <c r="C69" s="13" t="inlineStr">
+        <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D69" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E69" s="15" t="inlineStr">
+      <c r="E69" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2510,7 +2587,7 @@
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>Galería "en vivo"</t>
+          <t>Encabezado (hero)</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
@@ -2525,6 +2602,60 @@
       </c>
       <c r="F70" s="11" t="inlineStr"/>
       <c r="G70" s="11" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="B71" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C71" s="9" t="inlineStr">
+        <is>
+          <t>En qué consiste (card)</t>
+        </is>
+      </c>
+      <c r="D71" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E71" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F71" s="11" t="inlineStr"/>
+      <c r="G71" s="11" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="B72" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C72" s="9" t="inlineStr">
+        <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D72" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E72" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F72" s="11" t="inlineStr"/>
+      <c r="G72" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Bingo Show: portada con 3 fotos (flechas+logos+velo como home), card y galeria con fotos reales; inventario Bingo Show actualizado (7 fotos + link carpeta)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventario-fotos-web.xlsx
+++ b/inventario-fotos-web.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1360,7 +1360,6 @@
           <t>https://drive.google.com/drive/folders/1YutPNgTVrT9IIkybRK9farlrShKlAHCo</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="12" t="n">
@@ -1396,7 +1395,6 @@
           <t>https://drive.google.com/drive/folders/1YutPNgTVrT9IIkybRK9farlrShKlAHCo</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="12" t="n">
@@ -1512,7 +1510,6 @@
           <t>https://drive.google.com/drive/folders/1YutPNgTVrT9IIkybRK9farlrShKlAHCo</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="12" t="n">
@@ -1548,7 +1545,6 @@
           <t>https://drive.google.com/drive/folders/1YutPNgTVrT9IIkybRK9farlrShKlAHCo</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="12" t="n">
@@ -2349,16 +2345,25 @@
       </c>
       <c r="D61" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Día del Trabajador — presentador con micrófono y tablero BINGO</t>
         </is>
       </c>
       <c r="E61" s="16" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F61" s="11" t="inlineStr"/>
-      <c r="G61" s="11" t="inlineStr"/>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F61" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G61" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="12" t="n">
@@ -2371,21 +2376,30 @@
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>En qué consiste (card)</t>
+          <t>Encabezado (hero)</t>
         </is>
       </c>
       <c r="D62" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Almuerzo corporativo — banquete montado en el jardín</t>
         </is>
       </c>
       <c r="E62" s="16" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F62" s="11" t="inlineStr"/>
-      <c r="G62" s="11" t="inlineStr"/>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F62" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G62" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="12" t="n">
@@ -2398,102 +2412,138 @@
       </c>
       <c r="C63" s="13" t="inlineStr">
         <is>
+          <t>Encabezado (hero)</t>
+        </is>
+      </c>
+      <c r="D63" s="13" t="inlineStr">
+        <is>
+          <t>Bingo Show en el jardín — pelotitas azules</t>
+        </is>
+      </c>
+      <c r="E63" s="16" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F63" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G63" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="12" t="n">
+        <v>58</v>
+      </c>
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>Bingo Show (subpágina)</t>
+        </is>
+      </c>
+      <c r="C64" s="13" t="inlineStr">
+        <is>
+          <t>En qué consiste (card)</t>
+        </is>
+      </c>
+      <c r="D64" s="13" t="inlineStr">
+        <is>
+          <t>Pelotitas en primer plano con multitud de colaboradores detrás</t>
+        </is>
+      </c>
+      <c r="E64" s="16" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F64" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G64" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="n">
+        <v>59</v>
+      </c>
+      <c r="B65" s="13" t="inlineStr">
+        <is>
+          <t>Bingo Show (subpágina)</t>
+        </is>
+      </c>
+      <c r="C65" s="13" t="inlineStr">
+        <is>
           <t>Galería "en vivo"</t>
         </is>
       </c>
-      <c r="D63" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E63" s="16" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F63" s="11" t="inlineStr"/>
-      <c r="G63" s="11" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="8" t="n">
-        <v>58</v>
-      </c>
-      <c r="B64" s="9" t="inlineStr">
-        <is>
-          <t>Juegos de feria (subpágina)</t>
-        </is>
-      </c>
-      <c r="C64" s="9" t="inlineStr">
-        <is>
-          <t>Encabezado (hero)</t>
-        </is>
-      </c>
-      <c r="D64" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E64" s="15" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F64" s="11" t="inlineStr"/>
-      <c r="G64" s="11" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="8" t="n">
-        <v>59</v>
-      </c>
-      <c r="B65" s="9" t="inlineStr">
-        <is>
-          <t>Juegos de feria (subpágina)</t>
-        </is>
-      </c>
-      <c r="C65" s="9" t="inlineStr">
-        <is>
-          <t>En qué consiste (card)</t>
-        </is>
-      </c>
-      <c r="D65" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E65" s="15" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F65" s="11" t="inlineStr"/>
-      <c r="G65" s="11" t="inlineStr"/>
+      <c r="D65" s="13" t="inlineStr">
+        <is>
+          <t>Presentadores (traje rojo / vestido rosado) con bombo de bingo</t>
+        </is>
+      </c>
+      <c r="E65" s="16" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F65" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G65" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="8" t="n">
+      <c r="A66" s="12" t="n">
         <v>60</v>
       </c>
-      <c r="B66" s="9" t="inlineStr">
-        <is>
-          <t>Juegos de feria (subpágina)</t>
-        </is>
-      </c>
-      <c r="C66" s="9" t="inlineStr">
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>Bingo Show (subpágina)</t>
+        </is>
+      </c>
+      <c r="C66" s="13" t="inlineStr">
         <is>
           <t>Galería "en vivo"</t>
         </is>
       </c>
-      <c r="D66" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E66" s="15" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F66" s="11" t="inlineStr"/>
-      <c r="G66" s="11" t="inlineStr"/>
+      <c r="D66" s="13" t="inlineStr">
+        <is>
+          <t>Montaje de Bingo Show (Grupo National)</t>
+        </is>
+      </c>
+      <c r="E66" s="16" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F66" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G66" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="12" t="n">
@@ -2501,47 +2551,56 @@
       </c>
       <c r="B67" s="13" t="inlineStr">
         <is>
-          <t>Full Day (subpágina)</t>
+          <t>Bingo Show (subpágina)</t>
         </is>
       </c>
       <c r="C67" s="13" t="inlineStr">
         <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D67" s="13" t="inlineStr">
+        <is>
+          <t>Grupo posando con carteles (Día del Trabajador)</t>
+        </is>
+      </c>
+      <c r="E67" s="16" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F67" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G67" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="n">
+        <v>62</v>
+      </c>
+      <c r="B68" s="9" t="inlineStr">
+        <is>
+          <t>Juegos de feria (subpágina)</t>
+        </is>
+      </c>
+      <c r="C68" s="9" t="inlineStr">
+        <is>
           <t>Encabezado (hero)</t>
         </is>
       </c>
-      <c r="D67" s="13" t="inlineStr">
+      <c r="D68" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E67" s="16" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F67" s="11" t="inlineStr"/>
-      <c r="G67" s="11" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="12" t="n">
-        <v>62</v>
-      </c>
-      <c r="B68" s="13" t="inlineStr">
-        <is>
-          <t>Full Day (subpágina)</t>
-        </is>
-      </c>
-      <c r="C68" s="13" t="inlineStr">
-        <is>
-          <t>En qué consiste (card)</t>
-        </is>
-      </c>
-      <c r="D68" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E68" s="16" t="inlineStr">
+      <c r="E68" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2550,25 +2609,25 @@
       <c r="G68" s="11" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="12" t="n">
+      <c r="A69" s="8" t="n">
         <v>63</v>
       </c>
-      <c r="B69" s="13" t="inlineStr">
-        <is>
-          <t>Full Day (subpágina)</t>
-        </is>
-      </c>
-      <c r="C69" s="13" t="inlineStr">
-        <is>
-          <t>Galería "en vivo"</t>
-        </is>
-      </c>
-      <c r="D69" s="13" t="inlineStr">
+      <c r="B69" s="9" t="inlineStr">
+        <is>
+          <t>Juegos de feria (subpágina)</t>
+        </is>
+      </c>
+      <c r="C69" s="9" t="inlineStr">
+        <is>
+          <t>En qué consiste (card)</t>
+        </is>
+      </c>
+      <c r="D69" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E69" s="16" t="inlineStr">
+      <c r="E69" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2582,12 +2641,12 @@
       </c>
       <c r="B70" s="9" t="inlineStr">
         <is>
-          <t>Eventos privados (subpágina)</t>
+          <t>Juegos de feria (subpágina)</t>
         </is>
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>Encabezado (hero)</t>
+          <t>Galería "en vivo"</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
@@ -2604,25 +2663,25 @@
       <c r="G70" s="11" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="8" t="n">
+      <c r="A71" s="12" t="n">
         <v>65</v>
       </c>
-      <c r="B71" s="9" t="inlineStr">
-        <is>
-          <t>Eventos privados (subpágina)</t>
-        </is>
-      </c>
-      <c r="C71" s="9" t="inlineStr">
-        <is>
-          <t>En qué consiste (card)</t>
-        </is>
-      </c>
-      <c r="D71" s="9" t="inlineStr">
+      <c r="B71" s="13" t="inlineStr">
+        <is>
+          <t>Full Day (subpágina)</t>
+        </is>
+      </c>
+      <c r="C71" s="13" t="inlineStr">
+        <is>
+          <t>Encabezado (hero)</t>
+        </is>
+      </c>
+      <c r="D71" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E71" s="15" t="inlineStr">
+      <c r="E71" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2631,31 +2690,139 @@
       <c r="G71" s="11" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="8" t="n">
+      <c r="A72" s="12" t="n">
         <v>66</v>
       </c>
-      <c r="B72" s="9" t="inlineStr">
-        <is>
-          <t>Eventos privados (subpágina)</t>
-        </is>
-      </c>
-      <c r="C72" s="9" t="inlineStr">
-        <is>
-          <t>Galería "en vivo"</t>
-        </is>
-      </c>
-      <c r="D72" s="9" t="inlineStr">
+      <c r="B72" s="13" t="inlineStr">
+        <is>
+          <t>Full Day (subpágina)</t>
+        </is>
+      </c>
+      <c r="C72" s="13" t="inlineStr">
+        <is>
+          <t>En qué consiste (card)</t>
+        </is>
+      </c>
+      <c r="D72" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E72" s="15" t="inlineStr">
+      <c r="E72" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
       <c r="F72" s="11" t="inlineStr"/>
       <c r="G72" s="11" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="12" t="n">
+        <v>67</v>
+      </c>
+      <c r="B73" s="13" t="inlineStr">
+        <is>
+          <t>Full Day (subpágina)</t>
+        </is>
+      </c>
+      <c r="C73" s="13" t="inlineStr">
+        <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D73" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E73" s="16" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F73" s="11" t="inlineStr"/>
+      <c r="G73" s="11" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="n">
+        <v>68</v>
+      </c>
+      <c r="B74" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C74" s="9" t="inlineStr">
+        <is>
+          <t>Encabezado (hero)</t>
+        </is>
+      </c>
+      <c r="D74" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E74" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F74" s="11" t="inlineStr"/>
+      <c r="G74" s="11" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="B75" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C75" s="9" t="inlineStr">
+        <is>
+          <t>En qué consiste (card)</t>
+        </is>
+      </c>
+      <c r="D75" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E75" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F75" s="11" t="inlineStr"/>
+      <c r="G75" s="11" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="B76" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C76" s="9" t="inlineStr">
+        <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D76" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E76" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F76" s="11" t="inlineStr"/>
+      <c r="G76" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Team-building: card de resultados solo jovenes (quita señores); portada con flechas+logos como home; galeria imagen unica rotativa. Bingo Show: galeria imagen unica rotativa+flechas. Inventario actualizado
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventario-fotos-web.xlsx
+++ b/inventario-fotos-web.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2102,7 +2102,7 @@
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>Foto 1</t>
+          <t>Jóvenes en círculo — dinámica de manos (team building)</t>
         </is>
       </c>
       <c r="E52" s="14" t="inlineStr">
@@ -2124,12 +2124,12 @@
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>En qué consiste (card vertical)</t>
+          <t>Galería "en acción" (carrusel)</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
         <is>
-          <t>Foto 2</t>
+          <t>Foto 1</t>
         </is>
       </c>
       <c r="E53" s="14" t="inlineStr">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="D54" s="13" t="inlineStr">
         <is>
-          <t>Foto 1</t>
+          <t>Foto 2</t>
         </is>
       </c>
       <c r="E54" s="14" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="D55" s="13" t="inlineStr">
         <is>
-          <t>Foto 2</t>
+          <t>Foto 3</t>
         </is>
       </c>
       <c r="E55" s="14" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="D56" s="13" t="inlineStr">
         <is>
-          <t>Foto 3</t>
+          <t>Foto 4</t>
         </is>
       </c>
       <c r="E56" s="14" t="inlineStr">
@@ -2222,27 +2222,27 @@
       <c r="G56" s="11" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="12" t="n">
+      <c r="A57" s="8" t="n">
         <v>51</v>
       </c>
-      <c r="B57" s="13" t="inlineStr">
-        <is>
-          <t>Team building (subpágina)</t>
-        </is>
-      </c>
-      <c r="C57" s="13" t="inlineStr">
-        <is>
-          <t>Galería "en acción" (carrusel)</t>
-        </is>
-      </c>
-      <c r="D57" s="13" t="inlineStr">
-        <is>
-          <t>Foto 4</t>
-        </is>
-      </c>
-      <c r="E57" s="14" t="inlineStr">
-        <is>
-          <t>Cargada</t>
+      <c r="B57" s="9" t="inlineStr">
+        <is>
+          <t>Gymkanas productivas (subpágina)</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>Encabezado (hero)</t>
+        </is>
+      </c>
+      <c r="D57" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E57" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F57" s="11" t="inlineStr"/>
@@ -2259,7 +2259,7 @@
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>Encabezado (hero)</t>
+          <t>En qué consiste (card)</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>En qué consiste (card)</t>
+          <t>Galería "en vivo"</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
@@ -2303,31 +2303,39 @@
       <c r="G59" s="11" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="8" t="n">
+      <c r="A60" s="12" t="n">
         <v>54</v>
       </c>
-      <c r="B60" s="9" t="inlineStr">
-        <is>
-          <t>Gymkanas productivas (subpágina)</t>
-        </is>
-      </c>
-      <c r="C60" s="9" t="inlineStr">
-        <is>
-          <t>Galería "en vivo"</t>
-        </is>
-      </c>
-      <c r="D60" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E60" s="15" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F60" s="11" t="inlineStr"/>
-      <c r="G60" s="11" t="inlineStr"/>
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>Bingo Show (subpágina)</t>
+        </is>
+      </c>
+      <c r="C60" s="13" t="inlineStr">
+        <is>
+          <t>Encabezado (hero)</t>
+        </is>
+      </c>
+      <c r="D60" s="13" t="inlineStr">
+        <is>
+          <t>Día del Trabajador — presentador con micrófono y tablero BINGO</t>
+        </is>
+      </c>
+      <c r="E60" s="16" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F60" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G60" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="12" t="n">
@@ -2345,7 +2353,7 @@
       </c>
       <c r="D61" s="13" t="inlineStr">
         <is>
-          <t>Día del Trabajador — presentador con micrófono y tablero BINGO</t>
+          <t>Almuerzo corporativo — banquete montado en el jardín</t>
         </is>
       </c>
       <c r="E61" s="16" t="inlineStr">
@@ -2363,7 +2371,6 @@
           <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="12" t="n">
@@ -2381,7 +2388,7 @@
       </c>
       <c r="D62" s="13" t="inlineStr">
         <is>
-          <t>Almuerzo corporativo — banquete montado en el jardín</t>
+          <t>Bingo Show en el jardín — pelotitas azules</t>
         </is>
       </c>
       <c r="E62" s="16" t="inlineStr">
@@ -2399,7 +2406,6 @@
           <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="12" t="n">
@@ -2412,12 +2418,12 @@
       </c>
       <c r="C63" s="13" t="inlineStr">
         <is>
-          <t>Encabezado (hero)</t>
+          <t>En qué consiste (card)</t>
         </is>
       </c>
       <c r="D63" s="13" t="inlineStr">
         <is>
-          <t>Bingo Show en el jardín — pelotitas azules</t>
+          <t>Pelotitas en primer plano con multitud de colaboradores detrás</t>
         </is>
       </c>
       <c r="E63" s="16" t="inlineStr">
@@ -2435,7 +2441,6 @@
           <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="12" t="n">
@@ -2448,12 +2453,12 @@
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>En qué consiste (card)</t>
+          <t>Galería "en vivo"</t>
         </is>
       </c>
       <c r="D64" s="13" t="inlineStr">
         <is>
-          <t>Pelotitas en primer plano con multitud de colaboradores detrás</t>
+          <t>Presentadores (traje rojo / vestido rosado) con bombo de bingo</t>
         </is>
       </c>
       <c r="E64" s="16" t="inlineStr">
@@ -2471,7 +2476,6 @@
           <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="12" t="n">
@@ -2489,7 +2493,7 @@
       </c>
       <c r="D65" s="13" t="inlineStr">
         <is>
-          <t>Presentadores (traje rojo / vestido rosado) con bombo de bingo</t>
+          <t>Montaje de Bingo Show (Grupo National)</t>
         </is>
       </c>
       <c r="E65" s="16" t="inlineStr">
@@ -2507,7 +2511,6 @@
           <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="12" t="n">
@@ -2525,7 +2528,7 @@
       </c>
       <c r="D66" s="13" t="inlineStr">
         <is>
-          <t>Montaje de Bingo Show (Grupo National)</t>
+          <t>Grupo posando con carteles (Día del Trabajador)</t>
         </is>
       </c>
       <c r="E66" s="16" t="inlineStr">
@@ -2543,43 +2546,33 @@
           <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="12" t="n">
+      <c r="A67" s="8" t="n">
         <v>61</v>
       </c>
-      <c r="B67" s="13" t="inlineStr">
-        <is>
-          <t>Bingo Show (subpágina)</t>
-        </is>
-      </c>
-      <c r="C67" s="13" t="inlineStr">
-        <is>
-          <t>Galería "en vivo"</t>
-        </is>
-      </c>
-      <c r="D67" s="13" t="inlineStr">
-        <is>
-          <t>Grupo posando con carteles (Día del Trabajador)</t>
-        </is>
-      </c>
-      <c r="E67" s="16" t="inlineStr">
-        <is>
-          <t>Cargada</t>
-        </is>
-      </c>
-      <c r="F67" s="22" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G67" s="24" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr"/>
+      <c r="B67" s="9" t="inlineStr">
+        <is>
+          <t>Juegos de feria (subpágina)</t>
+        </is>
+      </c>
+      <c r="C67" s="9" t="inlineStr">
+        <is>
+          <t>Encabezado (hero)</t>
+        </is>
+      </c>
+      <c r="D67" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E67" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F67" s="11" t="inlineStr"/>
+      <c r="G67" s="11" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="8" t="n">
@@ -2592,7 +2585,7 @@
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>Encabezado (hero)</t>
+          <t>En qué consiste (card)</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
@@ -2619,7 +2612,7 @@
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>En qué consiste (card)</t>
+          <t>Galería "en vivo"</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
@@ -2636,25 +2629,25 @@
       <c r="G69" s="11" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="8" t="n">
+      <c r="A70" s="12" t="n">
         <v>64</v>
       </c>
-      <c r="B70" s="9" t="inlineStr">
-        <is>
-          <t>Juegos de feria (subpágina)</t>
-        </is>
-      </c>
-      <c r="C70" s="9" t="inlineStr">
-        <is>
-          <t>Galería "en vivo"</t>
-        </is>
-      </c>
-      <c r="D70" s="9" t="inlineStr">
+      <c r="B70" s="13" t="inlineStr">
+        <is>
+          <t>Full Day (subpágina)</t>
+        </is>
+      </c>
+      <c r="C70" s="13" t="inlineStr">
+        <is>
+          <t>Encabezado (hero)</t>
+        </is>
+      </c>
+      <c r="D70" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E70" s="15" t="inlineStr">
+      <c r="E70" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2673,7 +2666,7 @@
       </c>
       <c r="C71" s="13" t="inlineStr">
         <is>
-          <t>Encabezado (hero)</t>
+          <t>En qué consiste (card)</t>
         </is>
       </c>
       <c r="D71" s="13" t="inlineStr">
@@ -2700,7 +2693,7 @@
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>En qué consiste (card)</t>
+          <t>Galería "en vivo"</t>
         </is>
       </c>
       <c r="D72" s="13" t="inlineStr">
@@ -2717,25 +2710,25 @@
       <c r="G72" s="11" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="12" t="n">
+      <c r="A73" s="8" t="n">
         <v>67</v>
       </c>
-      <c r="B73" s="13" t="inlineStr">
-        <is>
-          <t>Full Day (subpágina)</t>
-        </is>
-      </c>
-      <c r="C73" s="13" t="inlineStr">
-        <is>
-          <t>Galería "en vivo"</t>
-        </is>
-      </c>
-      <c r="D73" s="13" t="inlineStr">
+      <c r="B73" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C73" s="9" t="inlineStr">
+        <is>
+          <t>Encabezado (hero)</t>
+        </is>
+      </c>
+      <c r="D73" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E73" s="16" t="inlineStr">
+      <c r="E73" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2754,7 +2747,7 @@
       </c>
       <c r="C74" s="9" t="inlineStr">
         <is>
-          <t>Encabezado (hero)</t>
+          <t>En qué consiste (card)</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
@@ -2781,7 +2774,7 @@
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>En qué consiste (card)</t>
+          <t>Galería "en vivo"</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
@@ -2796,33 +2789,6 @@
       </c>
       <c r="F75" s="11" t="inlineStr"/>
       <c r="G75" s="11" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="8" t="n">
-        <v>70</v>
-      </c>
-      <c r="B76" s="9" t="inlineStr">
-        <is>
-          <t>Eventos privados (subpágina)</t>
-        </is>
-      </c>
-      <c r="C76" s="9" t="inlineStr">
-        <is>
-          <t>Galería "en vivo"</t>
-        </is>
-      </c>
-      <c r="D76" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E76" s="15" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F76" s="11" t="inlineStr"/>
-      <c r="G76" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Eventos Privados: portada 4 fotos (flechas+logos+velo), card resultados, galeria rotativa 7 fotos; card en experiencias.html; inventario actualizado
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventario-fotos-web.xlsx
+++ b/inventario-fotos-web.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1315,51 +1315,43 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
+          <t>Equipo de Team building Ravina</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="n"/>
+      <c r="G25" s="11" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Inicio</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Diferenciales</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
           <t>Equipo trabajando junto en actividad</t>
         </is>
       </c>
-      <c r="E25" s="10" t="inlineStr">
-        <is>
-          <t>Cargada</t>
-        </is>
-      </c>
-      <c r="F25" s="11" t="inlineStr"/>
-      <c r="G25" s="11" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="12" t="n">
-        <v>20</v>
-      </c>
-      <c r="B26" s="13" t="inlineStr">
-        <is>
-          <t>Quiénes somos</t>
-        </is>
-      </c>
-      <c r="C26" s="13" t="inlineStr">
-        <is>
-          <t>Encabezado (carrusel)</t>
-        </is>
-      </c>
-      <c r="D26" s="13" t="inlineStr">
-        <is>
-          <t>Colaboradores compartiendo en evento corporativo</t>
-        </is>
-      </c>
-      <c r="E26" s="14" t="inlineStr">
-        <is>
-          <t>Cargada</t>
-        </is>
-      </c>
-      <c r="F26" s="22" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G26" s="24" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1YutPNgTVrT9IIkybRK9farlrShKlAHCo</t>
-        </is>
-      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr"/>
+      <c r="G26" s="11" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="12" t="n">
@@ -1377,7 +1369,7 @@
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>Fútbol burbuja en el campo</t>
+          <t>Colaboradores compartiendo en evento corporativo</t>
         </is>
       </c>
       <c r="E27" s="14" t="inlineStr">
@@ -1412,7 +1404,7 @@
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>Batucada y comparsa corporativa</t>
+          <t>Fútbol burbuja en el campo</t>
         </is>
       </c>
       <c r="E28" s="14" t="inlineStr">
@@ -1428,11 +1420,6 @@
       <c r="G28" s="24" t="inlineStr">
         <is>
           <t>https://drive.google.com/drive/folders/1YutPNgTVrT9IIkybRK9farlrShKlAHCo</t>
-        </is>
-      </c>
-      <c r="H28" s="25" t="inlineStr">
-        <is>
-          <t>Se ve irreal (imagen IA)</t>
         </is>
       </c>
     </row>
@@ -1452,7 +1439,7 @@
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>Dinámica de disfraces en equipo</t>
+          <t>Batucada y comparsa corporativa</t>
         </is>
       </c>
       <c r="E29" s="14" t="inlineStr">
@@ -1492,7 +1479,7 @@
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Comedor del evento — mesas tipo picnic</t>
+          <t>Dinámica de disfraces en equipo</t>
         </is>
       </c>
       <c r="E30" s="14" t="inlineStr">
@@ -1508,6 +1495,11 @@
       <c r="G30" s="24" t="inlineStr">
         <is>
           <t>https://drive.google.com/drive/folders/1YutPNgTVrT9IIkybRK9farlrShKlAHCo</t>
+        </is>
+      </c>
+      <c r="H30" s="25" t="inlineStr">
+        <is>
+          <t>Se ve irreal (imagen IA)</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1519,7 @@
       </c>
       <c r="D31" s="13" t="inlineStr">
         <is>
-          <t>Estación de jugos y desayuno de feria</t>
+          <t>Comedor del evento — mesas tipo picnic</t>
         </is>
       </c>
       <c r="E31" s="14" t="inlineStr">
@@ -1557,12 +1549,12 @@
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Liderazgo</t>
+          <t>Encabezado (carrusel)</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>Foto de la pestaña</t>
+          <t>Estación de jugos y desayuno de feria</t>
         </is>
       </c>
       <c r="E32" s="14" t="inlineStr">
@@ -1570,8 +1562,16 @@
           <t>Cargada</t>
         </is>
       </c>
-      <c r="F32" s="11" t="inlineStr"/>
-      <c r="G32" s="11" t="inlineStr"/>
+      <c r="F32" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G32" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1YutPNgTVrT9IIkybRK9farlrShKlAHCo</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="12" t="n">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Productividad</t>
+          <t>Superpoderes — Liderazgo</t>
         </is>
       </c>
       <c r="D33" s="13" t="inlineStr">
@@ -1611,7 +1611,7 @@
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Engagement</t>
+          <t>Superpoderes — Productividad</t>
         </is>
       </c>
       <c r="D34" s="13" t="inlineStr">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Retención de talento</t>
+          <t>Superpoderes — Engagement</t>
         </is>
       </c>
       <c r="D35" s="13" t="inlineStr">
@@ -1665,12 +1665,12 @@
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Superpoderes — Calidez humana</t>
+          <t>Superpoderes — Retención de talento</t>
         </is>
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>Equipo con cartel "Solo integrados..."</t>
+          <t>Foto de la pestaña</t>
         </is>
       </c>
       <c r="E36" s="14" t="inlineStr">
@@ -1682,25 +1682,25 @@
       <c r="G36" s="11" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="n">
+      <c r="A37" s="12" t="n">
         <v>31</v>
       </c>
-      <c r="B37" s="9" t="inlineStr">
-        <is>
-          <t>Servicios</t>
-        </is>
-      </c>
-      <c r="C37" s="9" t="inlineStr">
-        <is>
-          <t>Encabezado (carrusel)</t>
-        </is>
-      </c>
-      <c r="D37" s="9" t="inlineStr">
-        <is>
-          <t>Fútbol burbuja corporativo</t>
-        </is>
-      </c>
-      <c r="E37" s="10" t="inlineStr">
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Quiénes somos</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>Superpoderes — Calidez humana</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>Equipo con cartel "Solo integrados..."</t>
+        </is>
+      </c>
+      <c r="E37" s="14" t="inlineStr">
         <is>
           <t>Cargada</t>
         </is>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Arco de bienvenida Gymkanas</t>
+          <t>Fútbol burbuja corporativo</t>
         </is>
       </c>
       <c r="E38" s="10" t="inlineStr">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Dinámica de disfraces corporativa</t>
+          <t>Arco de bienvenida Gymkanas</t>
         </is>
       </c>
       <c r="E39" s="10" t="inlineStr">
@@ -1778,7 +1778,7 @@
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Comparsa y batucada en evento</t>
+          <t>Dinámica de disfraces corporativa</t>
         </is>
       </c>
       <c r="E40" s="10" t="inlineStr">
@@ -1800,12 +1800,12 @@
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Gymkanas productivas</t>
+          <t>Encabezado (carrusel)</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Foto de la experiencia</t>
+          <t>Comparsa y batucada en evento</t>
         </is>
       </c>
       <c r="E41" s="10" t="inlineStr">
@@ -1827,7 +1827,7 @@
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Team building</t>
+          <t>Pestaña — Gymkanas productivas</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Bingo Show</t>
+          <t>Pestaña — Team building</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
@@ -1881,7 +1881,7 @@
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Juegos de feria</t>
+          <t>Pestaña — Bingo Show</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Full Day</t>
+          <t>Pestaña — Juegos de feria</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Pestaña — Eventos privados</t>
+          <t>Pestaña — Full Day</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
@@ -1952,25 +1952,25 @@
       <c r="G46" s="11" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="12" t="n">
+      <c r="A47" s="8" t="n">
         <v>41</v>
       </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>Team building (subpágina)</t>
-        </is>
-      </c>
-      <c r="C47" s="13" t="inlineStr">
-        <is>
-          <t>Encabezado (carrusel horizontal)</t>
-        </is>
-      </c>
-      <c r="D47" s="13" t="inlineStr">
-        <is>
-          <t>Foto 1</t>
-        </is>
-      </c>
-      <c r="E47" s="14" t="inlineStr">
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Pestaña — Eventos privados</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>Foto de la experiencia</t>
+        </is>
+      </c>
+      <c r="E47" s="10" t="inlineStr">
         <is>
           <t>Cargada</t>
         </is>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>Foto 2</t>
+          <t>Foto 1</t>
         </is>
       </c>
       <c r="E48" s="14" t="inlineStr">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="D49" s="13" t="inlineStr">
         <is>
-          <t>Foto 3</t>
+          <t>Foto 2</t>
         </is>
       </c>
       <c r="E49" s="14" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="D50" s="13" t="inlineStr">
         <is>
-          <t>Foto 4</t>
+          <t>Foto 3</t>
         </is>
       </c>
       <c r="E50" s="14" t="inlineStr">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>Foto 5</t>
+          <t>Foto 4</t>
         </is>
       </c>
       <c r="E51" s="14" t="inlineStr">
@@ -2097,12 +2097,12 @@
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>En qué consiste (card vertical)</t>
+          <t>Encabezado (carrusel horizontal)</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>Jóvenes en círculo — dinámica de manos (team building)</t>
+          <t>Foto 5</t>
         </is>
       </c>
       <c r="E52" s="14" t="inlineStr">
@@ -2124,12 +2124,12 @@
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>Galería "en acción" (carrusel)</t>
+          <t>En qué consiste (card vertical)</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
         <is>
-          <t>Foto 1</t>
+          <t>Jóvenes en círculo — dinámica de manos (team building)</t>
         </is>
       </c>
       <c r="E53" s="14" t="inlineStr">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="D54" s="13" t="inlineStr">
         <is>
-          <t>Foto 2</t>
+          <t>Foto 1</t>
         </is>
       </c>
       <c r="E54" s="14" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="D55" s="13" t="inlineStr">
         <is>
-          <t>Foto 3</t>
+          <t>Foto 2</t>
         </is>
       </c>
       <c r="E55" s="14" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="D56" s="13" t="inlineStr">
         <is>
-          <t>Foto 4</t>
+          <t>Foto 3</t>
         </is>
       </c>
       <c r="E56" s="14" t="inlineStr">
@@ -2222,27 +2222,27 @@
       <c r="G56" s="11" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="8" t="n">
+      <c r="A57" s="12" t="n">
         <v>51</v>
       </c>
-      <c r="B57" s="9" t="inlineStr">
-        <is>
-          <t>Gymkanas productivas (subpágina)</t>
-        </is>
-      </c>
-      <c r="C57" s="9" t="inlineStr">
-        <is>
-          <t>Encabezado (hero)</t>
-        </is>
-      </c>
-      <c r="D57" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E57" s="15" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>Team building (subpágina)</t>
+        </is>
+      </c>
+      <c r="C57" s="13" t="inlineStr">
+        <is>
+          <t>Galería "en acción" (carrusel)</t>
+        </is>
+      </c>
+      <c r="D57" s="13" t="inlineStr">
+        <is>
+          <t>Foto 4</t>
+        </is>
+      </c>
+      <c r="E57" s="14" t="inlineStr">
+        <is>
+          <t>Cargada</t>
         </is>
       </c>
       <c r="F57" s="11" t="inlineStr"/>
@@ -2259,7 +2259,7 @@
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>En qué consiste (card)</t>
+          <t>Encabezado (hero)</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>Galería "en vivo"</t>
+          <t>En qué consiste (card)</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
@@ -2303,39 +2303,31 @@
       <c r="G59" s="11" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="12" t="n">
+      <c r="A60" s="8" t="n">
         <v>54</v>
       </c>
-      <c r="B60" s="13" t="inlineStr">
-        <is>
-          <t>Bingo Show (subpágina)</t>
-        </is>
-      </c>
-      <c r="C60" s="13" t="inlineStr">
-        <is>
-          <t>Encabezado (hero)</t>
-        </is>
-      </c>
-      <c r="D60" s="13" t="inlineStr">
-        <is>
-          <t>Día del Trabajador — presentador con micrófono y tablero BINGO</t>
-        </is>
-      </c>
-      <c r="E60" s="16" t="inlineStr">
-        <is>
-          <t>Cargada</t>
-        </is>
-      </c>
-      <c r="F60" s="22" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G60" s="24" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
-        </is>
-      </c>
+      <c r="B60" s="9" t="inlineStr">
+        <is>
+          <t>Gymkanas productivas (subpágina)</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D60" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E60" s="15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F60" s="11" t="inlineStr"/>
+      <c r="G60" s="11" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="12" t="n">
@@ -2353,7 +2345,7 @@
       </c>
       <c r="D61" s="13" t="inlineStr">
         <is>
-          <t>Almuerzo corporativo — banquete montado en el jardín</t>
+          <t>Día del Trabajador — presentador con micrófono y tablero BINGO</t>
         </is>
       </c>
       <c r="E61" s="16" t="inlineStr">
@@ -2388,7 +2380,7 @@
       </c>
       <c r="D62" s="13" t="inlineStr">
         <is>
-          <t>Bingo Show en el jardín — pelotitas azules</t>
+          <t>Almuerzo corporativo — banquete montado en el jardín</t>
         </is>
       </c>
       <c r="E62" s="16" t="inlineStr">
@@ -2418,12 +2410,12 @@
       </c>
       <c r="C63" s="13" t="inlineStr">
         <is>
-          <t>En qué consiste (card)</t>
+          <t>Encabezado (hero)</t>
         </is>
       </c>
       <c r="D63" s="13" t="inlineStr">
         <is>
-          <t>Pelotitas en primer plano con multitud de colaboradores detrás</t>
+          <t>Bingo Show en el jardín — pelotitas azules</t>
         </is>
       </c>
       <c r="E63" s="16" t="inlineStr">
@@ -2453,12 +2445,12 @@
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>Galería "en vivo"</t>
+          <t>En qué consiste (card)</t>
         </is>
       </c>
       <c r="D64" s="13" t="inlineStr">
         <is>
-          <t>Presentadores (traje rojo / vestido rosado) con bombo de bingo</t>
+          <t>Pelotitas en primer plano con multitud de colaboradores detrás</t>
         </is>
       </c>
       <c r="E64" s="16" t="inlineStr">
@@ -2493,7 +2485,7 @@
       </c>
       <c r="D65" s="13" t="inlineStr">
         <is>
-          <t>Montaje de Bingo Show (Grupo National)</t>
+          <t>Presentadores (traje rojo / vestido rosado) con bombo de bingo</t>
         </is>
       </c>
       <c r="E65" s="16" t="inlineStr">
@@ -2528,51 +2520,59 @@
       </c>
       <c r="D66" s="13" t="inlineStr">
         <is>
+          <t>Montaje de Bingo Show (Grupo National)</t>
+        </is>
+      </c>
+      <c r="E66" s="16" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F66" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G66" s="24" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="12" t="n">
+        <v>61</v>
+      </c>
+      <c r="B67" s="13" t="inlineStr">
+        <is>
+          <t>Bingo Show (subpágina)</t>
+        </is>
+      </c>
+      <c r="C67" s="13" t="inlineStr">
+        <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D67" s="13" t="inlineStr">
+        <is>
           <t>Grupo posando con carteles (Día del Trabajador)</t>
         </is>
       </c>
-      <c r="E66" s="16" t="inlineStr">
-        <is>
-          <t>Cargada</t>
-        </is>
-      </c>
-      <c r="F66" s="22" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="G66" s="24" t="inlineStr">
+      <c r="E67" s="16" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F67" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G67" s="24" t="inlineStr">
         <is>
           <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
         </is>
       </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="8" t="n">
-        <v>61</v>
-      </c>
-      <c r="B67" s="9" t="inlineStr">
-        <is>
-          <t>Juegos de feria (subpágina)</t>
-        </is>
-      </c>
-      <c r="C67" s="9" t="inlineStr">
-        <is>
-          <t>Encabezado (hero)</t>
-        </is>
-      </c>
-      <c r="D67" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E67" s="15" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F67" s="11" t="inlineStr"/>
-      <c r="G67" s="11" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="8" t="n">
@@ -2585,7 +2585,7 @@
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>En qué consiste (card)</t>
+          <t>Encabezado (hero)</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
@@ -2612,7 +2612,7 @@
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>Galería "en vivo"</t>
+          <t>En qué consiste (card)</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
@@ -2629,25 +2629,25 @@
       <c r="G69" s="11" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="12" t="n">
+      <c r="A70" s="8" t="n">
         <v>64</v>
       </c>
-      <c r="B70" s="13" t="inlineStr">
-        <is>
-          <t>Full Day (subpágina)</t>
-        </is>
-      </c>
-      <c r="C70" s="13" t="inlineStr">
-        <is>
-          <t>Encabezado (hero)</t>
-        </is>
-      </c>
-      <c r="D70" s="13" t="inlineStr">
+      <c r="B70" s="9" t="inlineStr">
+        <is>
+          <t>Juegos de feria (subpágina)</t>
+        </is>
+      </c>
+      <c r="C70" s="9" t="inlineStr">
+        <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D70" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E70" s="16" t="inlineStr">
+      <c r="E70" s="15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="C71" s="13" t="inlineStr">
         <is>
-          <t>En qué consiste (card)</t>
+          <t>Encabezado (hero)</t>
         </is>
       </c>
       <c r="D71" s="13" t="inlineStr">
@@ -2693,7 +2693,7 @@
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>Galería "en vivo"</t>
+          <t>En qué consiste (card)</t>
         </is>
       </c>
       <c r="D72" s="13" t="inlineStr">
@@ -2710,25 +2710,25 @@
       <c r="G72" s="11" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="8" t="n">
+      <c r="A73" s="12" t="n">
         <v>67</v>
       </c>
-      <c r="B73" s="9" t="inlineStr">
-        <is>
-          <t>Eventos privados (subpágina)</t>
-        </is>
-      </c>
-      <c r="C73" s="9" t="inlineStr">
-        <is>
-          <t>Encabezado (hero)</t>
-        </is>
-      </c>
-      <c r="D73" s="9" t="inlineStr">
+      <c r="B73" s="13" t="inlineStr">
+        <is>
+          <t>Full Day (subpágina)</t>
+        </is>
+      </c>
+      <c r="C73" s="13" t="inlineStr">
+        <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D73" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E73" s="15" t="inlineStr">
+      <c r="E73" s="16" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -2747,21 +2747,30 @@
       </c>
       <c r="C74" s="9" t="inlineStr">
         <is>
-          <t>En qué consiste (card)</t>
+          <t>Encabezado (hero)</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Colaboradores compartiendo en evento privado (sándwiches y café)</t>
         </is>
       </c>
       <c r="E74" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F74" s="11" t="inlineStr"/>
-      <c r="G74" s="11" t="inlineStr"/>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F74" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G74" s="11" t="inlineStr">
+        <is>
+          <t>Carpeta CORPORATIVOS (Drive)</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="8" t="n">
@@ -2774,21 +2783,390 @@
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
+          <t>Encabezado (hero)</t>
+        </is>
+      </c>
+      <c r="D75" s="9" t="inlineStr">
+        <is>
+          <t>Plato servido en evento corporativo (arroz con pollo)</t>
+        </is>
+      </c>
+      <c r="E75" s="15" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F75" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G75" s="11" t="inlineStr">
+        <is>
+          <t>Carpeta CORPORATIVOS (Drive)</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="B76" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C76" s="9" t="inlineStr">
+        <is>
+          <t>Encabezado (hero)</t>
+        </is>
+      </c>
+      <c r="D76" s="9" t="inlineStr">
+        <is>
+          <t>Toldos y celebración en el jardín</t>
+        </is>
+      </c>
+      <c r="E76" s="15" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F76" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G76" s="11" t="inlineStr">
+        <is>
+          <t>Carpeta CORPORATIVOS (Drive)</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="8" t="n">
+        <v>71</v>
+      </c>
+      <c r="B77" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C77" s="9" t="inlineStr">
+        <is>
+          <t>Encabezado (hero)</t>
+        </is>
+      </c>
+      <c r="D77" s="9" t="inlineStr">
+        <is>
+          <t>Banquete de pollo y papas al horno</t>
+        </is>
+      </c>
+      <c r="E77" s="15" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F77" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G77" s="11" t="inlineStr">
+        <is>
+          <t>Carpeta CORPORATIVOS (Drive)</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="8" t="n">
+        <v>72</v>
+      </c>
+      <c r="B78" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C78" s="9" t="inlineStr">
+        <is>
+          <t>En qué consiste (card)</t>
+        </is>
+      </c>
+      <c r="D78" s="9" t="inlineStr">
+        <is>
+          <t>Equipo celebrando con sombreros y globos</t>
+        </is>
+      </c>
+      <c r="E78" s="15" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F78" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G78" s="11" t="inlineStr">
+        <is>
+          <t>Carpeta CORPORATIVOS (Drive)</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="n">
+        <v>73</v>
+      </c>
+      <c r="B79" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C79" s="9" t="inlineStr">
+        <is>
           <t>Galería "en vivo"</t>
         </is>
       </c>
-      <c r="D75" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E75" s="15" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F75" s="11" t="inlineStr"/>
-      <c r="G75" s="11" t="inlineStr"/>
+      <c r="D79" s="9" t="inlineStr">
+        <is>
+          <t>Equipo de catering del evento</t>
+        </is>
+      </c>
+      <c r="E79" s="15" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F79" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G79" s="11" t="inlineStr">
+        <is>
+          <t>Carpeta CORPORATIVOS (Drive)</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="B80" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C80" s="9" t="inlineStr">
+        <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D80" s="9" t="inlineStr">
+        <is>
+          <t>Parrillas listas para el banquete</t>
+        </is>
+      </c>
+      <c r="E80" s="15" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F80" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G80" s="11" t="inlineStr">
+        <is>
+          <t>Carpeta CORPORATIVOS (Drive)</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="8" t="n">
+        <v>75</v>
+      </c>
+      <c r="B81" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C81" s="9" t="inlineStr">
+        <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D81" s="9" t="inlineStr">
+        <is>
+          <t>Cocinera sirviendo picarones</t>
+        </is>
+      </c>
+      <c r="E81" s="15" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F81" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G81" s="11" t="inlineStr">
+        <is>
+          <t>Carpeta CORPORATIVOS (Drive)</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="n">
+        <v>76</v>
+      </c>
+      <c r="B82" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C82" s="9" t="inlineStr">
+        <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D82" s="9" t="inlineStr">
+        <is>
+          <t>Invitada saludando bajo las sombrillas</t>
+        </is>
+      </c>
+      <c r="E82" s="15" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F82" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G82" s="11" t="inlineStr">
+        <is>
+          <t>Carpeta CORPORATIVOS (Drive)</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="8" t="n">
+        <v>77</v>
+      </c>
+      <c r="B83" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C83" s="9" t="inlineStr">
+        <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D83" s="9" t="inlineStr">
+        <is>
+          <t>Barra de mojitos en evento</t>
+        </is>
+      </c>
+      <c r="E83" s="15" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F83" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G83" s="11" t="inlineStr">
+        <is>
+          <t>Carpeta CORPORATIVOS (Drive)</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="B84" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C84" s="9" t="inlineStr">
+        <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D84" s="9" t="inlineStr">
+        <is>
+          <t>Colaboradores celebrando con trofeo</t>
+        </is>
+      </c>
+      <c r="E84" s="15" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F84" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G84" s="11" t="inlineStr">
+        <is>
+          <t>Carpeta CORPORATIVOS (Drive)</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="B85" s="9" t="inlineStr">
+        <is>
+          <t>Eventos privados (subpágina)</t>
+        </is>
+      </c>
+      <c r="C85" s="9" t="inlineStr">
+        <is>
+          <t>Galería "en vivo"</t>
+        </is>
+      </c>
+      <c r="D85" s="9" t="inlineStr">
+        <is>
+          <t>Picarones con miel</t>
+        </is>
+      </c>
+      <c r="E85" s="15" t="inlineStr">
+        <is>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F85" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G85" s="11" t="inlineStr">
+        <is>
+          <t>Carpeta CORPORATIVOS (Drive)</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Eventos Privados: intercambia foto de cocinera (a portada) y colaboradores (a galeria); inventario actualizado
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventario-fotos-web.xlsx
+++ b/inventario-fotos-web.xlsx
@@ -670,6 +670,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
@@ -2752,7 +2753,7 @@
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Colaboradores compartiendo en evento privado (sándwiches y café)</t>
+          <t>Cocinera sirviendo picarones</t>
         </is>
       </c>
       <c r="E74" s="15" t="inlineStr">
@@ -2770,7 +2771,6 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="8" t="n">
@@ -2806,7 +2806,6 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="8" t="n">
@@ -2842,7 +2841,6 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="8" t="n">
@@ -2878,7 +2876,6 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="8" t="n">
@@ -2914,7 +2911,6 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="8" t="n">
@@ -2950,7 +2946,6 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="8" t="n">
@@ -2986,7 +2981,6 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="8" t="n">
@@ -3004,7 +2998,7 @@
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Cocinera sirviendo picarones</t>
+          <t>Colaboradores compartiendo en evento privado (sándwiches y café)</t>
         </is>
       </c>
       <c r="E81" s="15" t="inlineStr">
@@ -3022,7 +3016,6 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="8" t="n">
@@ -3058,7 +3051,6 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="8" t="n">
@@ -3094,7 +3086,6 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="8" t="n">
@@ -3130,7 +3121,6 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="8" t="n">
@@ -3166,7 +3156,6 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Gymkanas productivas: portada con foto de gymkana de globos (velo + logos como las otras); carpeta de trabajo + inventario
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventario-fotos-web.xlsx
+++ b/inventario-fotos-web.xlsx
@@ -2265,16 +2265,24 @@
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Gymkana de globos — equipos comunicados (feria en jardín)</t>
         </is>
       </c>
       <c r="E58" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F58" s="11" t="inlineStr"/>
-      <c r="G58" s="11" t="inlineStr"/>
+          <t>Cargada</t>
+        </is>
+      </c>
+      <c r="F58" s="22" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G58" s="11" t="inlineStr">
+        <is>
+          <t>Carpeta GYMKANA YI CHANG</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="n">

</xml_diff>

<commit_message>
Inventario: portada Eventos Privados = foto del trofeo; cocinera picarones pasa a galeria (sincroniza con el sitio)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventario-fotos-web.xlsx
+++ b/inventario-fotos-web.xlsx
@@ -2761,7 +2761,7 @@
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Cocinera sirviendo picarones</t>
+          <t>Colaboradores celebrando con trofeo (mujer feliz levantando la copa)</t>
         </is>
       </c>
       <c r="E74" s="15" t="inlineStr">
@@ -2777,6 +2777,11 @@
       <c r="G74" s="11" t="inlineStr">
         <is>
           <t>Carpeta CORPORATIVOS (Drive)</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Movida desde la galería a la portada (2026-07-18)</t>
         </is>
       </c>
     </row>
@@ -3111,7 +3116,7 @@
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>Colaboradores celebrando con trofeo</t>
+          <t>Cocinera sirviendo picarones</t>
         </is>
       </c>
       <c r="E84" s="15" t="inlineStr">
@@ -3127,6 +3132,11 @@
       <c r="G84" s="11" t="inlineStr">
         <is>
           <t>Carpeta CORPORATIVOS (Drive)</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Bajada desde la portada a la galería (2026-07-18)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ruta /experiencias -> /servicios: renombra pagina y carpeta, actualiza todos los links internos
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventario-fotos-web.xlsx
+++ b/inventario-fotos-web.xlsx
@@ -192,7 +192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -261,6 +261,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -626,7 +629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:I85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -637,6 +640,7 @@
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -670,7 +674,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
@@ -712,6 +715,11 @@
           <t>Observación</t>
         </is>
       </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>¿Parece IA?</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -749,6 +757,7 @@
           <t>https://drive.google.com/...</t>
         </is>
       </c>
+      <c r="I6" s="26" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="20" t="n">
@@ -784,6 +793,7 @@
           <t>https://drive.google.com/file/d/1bpKGEEe5qZVCX2_WJ2bfcczSRdloF5gy/view</t>
         </is>
       </c>
+      <c r="I7" s="26" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="20" t="n">
@@ -819,6 +829,7 @@
           <t>https://drive.google.com/file/d/18gkDcpy2v4ajAHfLSjqStHPSv5znxVec/view</t>
         </is>
       </c>
+      <c r="I8" s="26" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="20" t="n">
@@ -854,6 +865,7 @@
           <t>https://drive.google.com/file/d/1IQIts1momeIJnvDenIN2V8zgI9Yuzu3I/view</t>
         </is>
       </c>
+      <c r="I9" s="26" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="20" t="n">
@@ -889,6 +901,7 @@
           <t>https://drive.google.com/file/d/11nmFeZH_GDXNDlBeqdOonSWJMttFoNm3/view</t>
         </is>
       </c>
+      <c r="I10" s="26" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n">
@@ -916,6 +929,7 @@
       </c>
       <c r="F11" s="11" t="inlineStr"/>
       <c r="G11" s="11" t="inlineStr"/>
+      <c r="I11" s="26" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
@@ -943,6 +957,7 @@
       </c>
       <c r="F12" s="11" t="inlineStr"/>
       <c r="G12" s="11" t="inlineStr"/>
+      <c r="I12" s="26" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="n">
@@ -970,6 +985,7 @@
       </c>
       <c r="F13" s="11" t="inlineStr"/>
       <c r="G13" s="11" t="inlineStr"/>
+      <c r="I13" s="26" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n">
@@ -1005,6 +1021,7 @@
           <t>https://drive.google.com/drive/folders/1CpiI8EKPfkVF_xjyozKN7ZMyFYGNK5xZ</t>
         </is>
       </c>
+      <c r="I14" s="26" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n">
@@ -1040,6 +1057,7 @@
           <t>https://drive.google.com/drive/folders/1CpiI8EKPfkVF_xjyozKN7ZMyFYGNK5xZ</t>
         </is>
       </c>
+      <c r="I15" s="26" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n">
@@ -1075,6 +1093,7 @@
           <t>https://drive.google.com/drive/folders/1CpiI8EKPfkVF_xjyozKN7ZMyFYGNK5xZ</t>
         </is>
       </c>
+      <c r="I16" s="26" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n">
@@ -1110,6 +1129,7 @@
           <t>https://drive.google.com/drive/folders/1CpiI8EKPfkVF_xjyozKN7ZMyFYGNK5xZ</t>
         </is>
       </c>
+      <c r="I17" s="26" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
@@ -1137,6 +1157,7 @@
       </c>
       <c r="F18" s="11" t="inlineStr"/>
       <c r="G18" s="11" t="inlineStr"/>
+      <c r="I18" s="26" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n">
@@ -1164,6 +1185,7 @@
       </c>
       <c r="F19" s="11" t="inlineStr"/>
       <c r="G19" s="11" t="inlineStr"/>
+      <c r="I19" s="26" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n">
@@ -1191,6 +1213,7 @@
       </c>
       <c r="F20" s="11" t="inlineStr"/>
       <c r="G20" s="11" t="inlineStr"/>
+      <c r="I20" s="26" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="n">
@@ -1218,6 +1241,7 @@
       </c>
       <c r="F21" s="11" t="inlineStr"/>
       <c r="G21" s="11" t="inlineStr"/>
+      <c r="I21" s="26" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n">
@@ -1245,6 +1269,7 @@
       </c>
       <c r="F22" s="11" t="inlineStr"/>
       <c r="G22" s="11" t="inlineStr"/>
+      <c r="I22" s="26" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="n">
@@ -1272,6 +1297,7 @@
       </c>
       <c r="F23" s="11" t="inlineStr"/>
       <c r="G23" s="11" t="inlineStr"/>
+      <c r="I23" s="26" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="8" t="n">
@@ -1299,6 +1325,7 @@
       </c>
       <c r="F24" s="11" t="inlineStr"/>
       <c r="G24" s="11" t="inlineStr"/>
+      <c r="I24" s="26" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="8" t="n">
@@ -1326,6 +1353,7 @@
       </c>
       <c r="F25" s="11" t="n"/>
       <c r="G25" s="11" t="n"/>
+      <c r="I25" s="26" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="n">
@@ -1353,6 +1381,7 @@
       </c>
       <c r="F26" s="11" t="inlineStr"/>
       <c r="G26" s="11" t="inlineStr"/>
+      <c r="I26" s="26" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="12" t="n">
@@ -1388,6 +1417,7 @@
           <t>https://drive.google.com/drive/folders/1YutPNgTVrT9IIkybRK9farlrShKlAHCo</t>
         </is>
       </c>
+      <c r="I27" s="26" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="12" t="n">
@@ -1423,6 +1453,7 @@
           <t>https://drive.google.com/drive/folders/1YutPNgTVrT9IIkybRK9farlrShKlAHCo</t>
         </is>
       </c>
+      <c r="I28" s="26" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="12" t="n">
@@ -1463,6 +1494,11 @@
           <t>Se ve irreal (imagen IA)</t>
         </is>
       </c>
+      <c r="I29" s="26" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="12" t="n">
@@ -1503,6 +1539,11 @@
           <t>Se ve irreal (imagen IA)</t>
         </is>
       </c>
+      <c r="I30" s="26" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="12" t="n">
@@ -1538,6 +1579,7 @@
           <t>https://drive.google.com/drive/folders/1YutPNgTVrT9IIkybRK9farlrShKlAHCo</t>
         </is>
       </c>
+      <c r="I31" s="26" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="12" t="n">
@@ -1573,6 +1615,7 @@
           <t>https://drive.google.com/drive/folders/1YutPNgTVrT9IIkybRK9farlrShKlAHCo</t>
         </is>
       </c>
+      <c r="I32" s="26" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="12" t="n">
@@ -1600,6 +1643,7 @@
       </c>
       <c r="F33" s="11" t="inlineStr"/>
       <c r="G33" s="11" t="inlineStr"/>
+      <c r="I33" s="26" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="12" t="n">
@@ -1627,6 +1671,7 @@
       </c>
       <c r="F34" s="11" t="inlineStr"/>
       <c r="G34" s="11" t="inlineStr"/>
+      <c r="I34" s="26" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="12" t="n">
@@ -1654,6 +1699,7 @@
       </c>
       <c r="F35" s="11" t="inlineStr"/>
       <c r="G35" s="11" t="inlineStr"/>
+      <c r="I35" s="26" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="12" t="n">
@@ -1681,6 +1727,7 @@
       </c>
       <c r="F36" s="11" t="inlineStr"/>
       <c r="G36" s="11" t="inlineStr"/>
+      <c r="I36" s="26" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="12" t="n">
@@ -1708,6 +1755,7 @@
       </c>
       <c r="F37" s="11" t="inlineStr"/>
       <c r="G37" s="11" t="inlineStr"/>
+      <c r="I37" s="26" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n">
@@ -1735,6 +1783,7 @@
       </c>
       <c r="F38" s="11" t="inlineStr"/>
       <c r="G38" s="11" t="inlineStr"/>
+      <c r="I38" s="26" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="8" t="n">
@@ -1762,6 +1811,7 @@
       </c>
       <c r="F39" s="11" t="inlineStr"/>
       <c r="G39" s="11" t="inlineStr"/>
+      <c r="I39" s="26" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="8" t="n">
@@ -1789,6 +1839,7 @@
       </c>
       <c r="F40" s="11" t="inlineStr"/>
       <c r="G40" s="11" t="inlineStr"/>
+      <c r="I40" s="26" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="8" t="n">
@@ -1816,6 +1867,7 @@
       </c>
       <c r="F41" s="11" t="inlineStr"/>
       <c r="G41" s="11" t="inlineStr"/>
+      <c r="I41" s="26" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="8" t="n">
@@ -1843,6 +1895,7 @@
       </c>
       <c r="F42" s="11" t="inlineStr"/>
       <c r="G42" s="11" t="inlineStr"/>
+      <c r="I42" s="26" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="8" t="n">
@@ -1870,6 +1923,7 @@
       </c>
       <c r="F43" s="11" t="inlineStr"/>
       <c r="G43" s="11" t="inlineStr"/>
+      <c r="I43" s="26" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="8" t="n">
@@ -1897,6 +1951,7 @@
       </c>
       <c r="F44" s="11" t="inlineStr"/>
       <c r="G44" s="11" t="inlineStr"/>
+      <c r="I44" s="26" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="8" t="n">
@@ -1924,6 +1979,7 @@
       </c>
       <c r="F45" s="11" t="inlineStr"/>
       <c r="G45" s="11" t="inlineStr"/>
+      <c r="I45" s="26" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="8" t="n">
@@ -1951,6 +2007,7 @@
       </c>
       <c r="F46" s="11" t="inlineStr"/>
       <c r="G46" s="11" t="inlineStr"/>
+      <c r="I46" s="26" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="8" t="n">
@@ -1978,6 +2035,7 @@
       </c>
       <c r="F47" s="11" t="inlineStr"/>
       <c r="G47" s="11" t="inlineStr"/>
+      <c r="I47" s="26" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="12" t="n">
@@ -2005,6 +2063,7 @@
       </c>
       <c r="F48" s="11" t="inlineStr"/>
       <c r="G48" s="11" t="inlineStr"/>
+      <c r="I48" s="26" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="12" t="n">
@@ -2032,6 +2091,7 @@
       </c>
       <c r="F49" s="11" t="inlineStr"/>
       <c r="G49" s="11" t="inlineStr"/>
+      <c r="I49" s="26" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="12" t="n">
@@ -2059,6 +2119,7 @@
       </c>
       <c r="F50" s="11" t="inlineStr"/>
       <c r="G50" s="11" t="inlineStr"/>
+      <c r="I50" s="26" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="12" t="n">
@@ -2086,6 +2147,7 @@
       </c>
       <c r="F51" s="11" t="inlineStr"/>
       <c r="G51" s="11" t="inlineStr"/>
+      <c r="I51" s="26" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="12" t="n">
@@ -2113,6 +2175,7 @@
       </c>
       <c r="F52" s="11" t="inlineStr"/>
       <c r="G52" s="11" t="inlineStr"/>
+      <c r="I52" s="26" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="12" t="n">
@@ -2140,6 +2203,7 @@
       </c>
       <c r="F53" s="11" t="inlineStr"/>
       <c r="G53" s="11" t="inlineStr"/>
+      <c r="I53" s="26" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="12" t="n">
@@ -2167,6 +2231,7 @@
       </c>
       <c r="F54" s="11" t="inlineStr"/>
       <c r="G54" s="11" t="inlineStr"/>
+      <c r="I54" s="26" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="12" t="n">
@@ -2194,6 +2259,7 @@
       </c>
       <c r="F55" s="11" t="inlineStr"/>
       <c r="G55" s="11" t="inlineStr"/>
+      <c r="I55" s="26" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="12" t="n">
@@ -2221,6 +2287,7 @@
       </c>
       <c r="F56" s="11" t="inlineStr"/>
       <c r="G56" s="11" t="inlineStr"/>
+      <c r="I56" s="26" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="12" t="n">
@@ -2248,6 +2315,7 @@
       </c>
       <c r="F57" s="11" t="inlineStr"/>
       <c r="G57" s="11" t="inlineStr"/>
+      <c r="I57" s="26" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="8" t="n">
@@ -2283,6 +2351,7 @@
           <t>Carpeta GYMKANA YI CHANG</t>
         </is>
       </c>
+      <c r="I58" s="26" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="8" t="n">
@@ -2310,6 +2379,7 @@
       </c>
       <c r="F59" s="11" t="inlineStr"/>
       <c r="G59" s="11" t="inlineStr"/>
+      <c r="I59" s="26" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="8" t="n">
@@ -2337,6 +2407,7 @@
       </c>
       <c r="F60" s="11" t="inlineStr"/>
       <c r="G60" s="11" t="inlineStr"/>
+      <c r="I60" s="26" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="12" t="n">
@@ -2372,6 +2443,7 @@
           <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
         </is>
       </c>
+      <c r="I61" s="26" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="12" t="n">
@@ -2407,6 +2479,7 @@
           <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
         </is>
       </c>
+      <c r="I62" s="26" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="12" t="n">
@@ -2442,6 +2515,7 @@
           <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
         </is>
       </c>
+      <c r="I63" s="26" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="12" t="n">
@@ -2477,6 +2551,7 @@
           <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
         </is>
       </c>
+      <c r="I64" s="26" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="12" t="n">
@@ -2512,6 +2587,7 @@
           <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
         </is>
       </c>
+      <c r="I65" s="26" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="12" t="n">
@@ -2547,6 +2623,7 @@
           <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
         </is>
       </c>
+      <c r="I66" s="26" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="12" t="n">
@@ -2582,6 +2659,7 @@
           <t>https://drive.google.com/drive/folders/1fA82mYG7KQ3OKAitRvHh_SQmhXthLpnm</t>
         </is>
       </c>
+      <c r="I67" s="26" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="8" t="n">
@@ -2609,6 +2687,7 @@
       </c>
       <c r="F68" s="11" t="inlineStr"/>
       <c r="G68" s="11" t="inlineStr"/>
+      <c r="I68" s="26" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="8" t="n">
@@ -2636,6 +2715,7 @@
       </c>
       <c r="F69" s="11" t="inlineStr"/>
       <c r="G69" s="11" t="inlineStr"/>
+      <c r="I69" s="26" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="8" t="n">
@@ -2663,6 +2743,7 @@
       </c>
       <c r="F70" s="11" t="inlineStr"/>
       <c r="G70" s="11" t="inlineStr"/>
+      <c r="I70" s="26" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="12" t="n">
@@ -2690,6 +2771,7 @@
       </c>
       <c r="F71" s="11" t="inlineStr"/>
       <c r="G71" s="11" t="inlineStr"/>
+      <c r="I71" s="26" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="12" t="n">
@@ -2717,6 +2799,7 @@
       </c>
       <c r="F72" s="11" t="inlineStr"/>
       <c r="G72" s="11" t="inlineStr"/>
+      <c r="I72" s="26" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="12" t="n">
@@ -2744,6 +2827,7 @@
       </c>
       <c r="F73" s="11" t="inlineStr"/>
       <c r="G73" s="11" t="inlineStr"/>
+      <c r="I73" s="26" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="8" t="n">
@@ -2784,6 +2868,7 @@
           <t>Movida desde la galería a la portada (2026-07-18)</t>
         </is>
       </c>
+      <c r="I74" s="26" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="8" t="n">
@@ -2819,6 +2904,7 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
+      <c r="I75" s="26" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="8" t="n">
@@ -2854,6 +2940,7 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
+      <c r="I76" s="26" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="8" t="n">
@@ -2889,6 +2976,7 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
+      <c r="I77" s="26" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="8" t="n">
@@ -2924,6 +3012,11 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
+      <c r="I78" s="26" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="n">
@@ -2959,6 +3052,7 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
+      <c r="I79" s="26" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="8" t="n">
@@ -2994,6 +3088,7 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
+      <c r="I80" s="26" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="8" t="n">
@@ -3029,6 +3124,7 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
+      <c r="I81" s="26" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="8" t="n">
@@ -3064,6 +3160,7 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
+      <c r="I82" s="26" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="8" t="n">
@@ -3099,6 +3196,7 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
+      <c r="I83" s="26" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="8" t="n">
@@ -3139,6 +3237,7 @@
           <t>Bajada desde la portada a la galería (2026-07-18)</t>
         </is>
       </c>
+      <c r="I84" s="26" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="8" t="n">
@@ -3174,6 +3273,7 @@
           <t>Carpeta CORPORATIVOS (Drive)</t>
         </is>
       </c>
+      <c r="I85" s="26" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>